<commit_message>
Update model to make compatible with de OSeMOSYS model version 5.4
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -1,28 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15FA81D0-8FC4-497D-83D3-B66A5A2D189D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A709DB37-B5A1-445B-B667-F0BF957A2960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{A38498C0-325E-4D75-9B65-6D8B75ECDFF0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
-    <sheet name="Setup" sheetId="2" r:id="rId2"/>
-    <sheet name="Params_Sets_Vari" sheetId="3" r:id="rId3"/>
-    <sheet name="To_Print" sheetId="4" r:id="rId4"/>
+    <sheet name="Uncertainty_Table" sheetId="13" r:id="rId1"/>
+    <sheet name="Setup" sheetId="3" r:id="rId2"/>
+    <sheet name="Params_Sets_Vari" sheetId="14" r:id="rId3"/>
+    <sheet name="To_Print" sheetId="12" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$O$40</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -44,17 +47,26 @@
     <author>Climate Lead Group</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{2F50FA3F-EF55-4802-9EDB-FD7396EEA55E}">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:
+          <t>Climate Lead Group:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Options:
 - Linear: Performs a linear interpolation starting at the year of “Initial_Year_of_Uncertainty” and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
 - Constant: Performs a constant curve starting at the year of “Initial_Year_of_Uncertainty” with its value and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
@@ -64,49 +76,76 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{4B113B91-8C7D-4026-9B16-B744A1863E43}">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:
+          <t>Climate Lead Group:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the first set of InputActivityRatio is t: TECHNOLOGY, so you need to put sets of TECHNOLOGY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{56220757-0F04-471C-A32C-C1D985AB505F}">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:
+          <t>Climate Lead Group:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the second set of InputActivityRatio is f: COMODDITY so you need to put sets of COMODDITY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{8E8A5497-9CD0-462C-9F22-242368490FCA}">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:
+          <t>Climate Lead Group:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the third set of InputActivityRatio is t: MODE_OF_OPERATION so you need to put sets of MODE_OF_OPERATION in this cell for that parameter.</t>
         </r>
@@ -122,17 +161,26 @@
     <author>Climate Lead Group</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{DBC5382B-8EB4-47E4-8B4B-119D1D2D7FE0}">
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:
+          <t>Climate Lead Group:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
 Parameters paint in brown can not do a variation in RDM experiment.</t>
         </r>
       </text>
@@ -142,7 +190,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="235">
   <si>
     <t>X_Num</t>
   </si>
@@ -189,39 +237,252 @@
     <t>Manipulation_of_Parameter</t>
   </si>
   <si>
+    <t>Demand Growth</t>
+  </si>
+  <si>
+    <t>Demand growth in the buildings sector</t>
+  </si>
+  <si>
+    <t>Scenario1</t>
+  </si>
+  <si>
+    <t>Time_Series</t>
+  </si>
+  <si>
+    <t>Final_Value</t>
+  </si>
+  <si>
+    <t>AccumulatedAnnualDemand</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>RESCKN ; RESLGT ; RESCOL ; RESWHT ; RESHEL ; RESELCOTH ; COMELCOTH ; COMHET ; TOURELCOTH ; TOURHET</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
+  </si>
+  <si>
+    <t>Demand growth in the industry sector</t>
+  </si>
+  <si>
+    <t>INDMIN ; INDASH ; INDCEM ; INDOTH</t>
+  </si>
+  <si>
+    <t>Demand growth in the transport sector</t>
+  </si>
+  <si>
+    <t>TRACAR ; TRAMCY ; TRABUS ; TRAMNB ; TRALTR ; TRAMTR ; TRAHTR ; TRARAILF ; TRAAVI</t>
+  </si>
+  <si>
+    <t>Capital Costs</t>
+  </si>
+  <si>
+    <t>Capital costs of electric vehicles</t>
+  </si>
+  <si>
+    <t>CapitalCost</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>TRAELCCARCUR ; TRAELCCARNEW ; TRAELCMCYCUR ; TRAELCMCYNEW ; TRAELCMNBCUR ; TRAELCMNBNEW ; TRAELCBUSCUR ; TRAELCBUSNEW ; TRAELCLTRCUR ; TRAELCLTRNEW ; TRAELCMTRCUR ; TRAELCMTRNEW ; TRAELCHTRCUR ; TRAELCHTRNEW</t>
+  </si>
+  <si>
+    <t>Fixed Costs</t>
+  </si>
+  <si>
+    <t>Fixed Cost of electric vehicles technologies</t>
+  </si>
+  <si>
+    <t>FixedCost</t>
+  </si>
+  <si>
+    <t>Capital Cost of ICE vehicles technologies</t>
+  </si>
+  <si>
+    <t>TRADSLCARCUR ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
+  </si>
+  <si>
+    <t>Fixed Cost of ICE vehicles technologies</t>
+  </si>
+  <si>
+    <t>Variable Costs</t>
+  </si>
+  <si>
+    <t>Variable Cost of crops technologies</t>
+  </si>
+  <si>
+    <t>VariableCost</t>
+  </si>
+  <si>
+    <t>LNDMAIHR ; LNDMAIHI ; LNDMAILR ; LNDMAILI ; LNDCANHR ; LNDCANHI ; LNDCANLR ; LNDCANLI ; LNDGROHR ; LNDGROHI ; LNDGROLR ; LNDGROLI ; LNDMTPHR ; LNDMTPHI ; LNDMTPLR ; LNDMTPLI ; LNDOTCHR ; LNDOTCHI ; LNDOTCLR ; LNDOTCLI ; LNDPULHR ; LNDPULHI ; LNDPULLR ; LNDPULLI ; LNDSORHR ; LNDSORHI ; LNDSORLR ; LNDSORLI ; LNDWHEHR ; LNDWHEHI ; LNDWHELR ; LNDWHELI</t>
+  </si>
+  <si>
+    <t>Fixed Cost of crops technologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import cost of fuels </t>
+  </si>
+  <si>
+    <t>IMPBIO ; IMPLPG ; IMPHFO ; IMPNGS ; IMPURN ; IMPGSL ; IMPDSL ; IMPKER</t>
+  </si>
+  <si>
+    <t>Cost of electricity imports</t>
+  </si>
+  <si>
+    <t>PWRTRNIMP</t>
+  </si>
+  <si>
+    <t>Cost of crop imports</t>
+  </si>
+  <si>
+    <t>IMPMAI ; IMPPUL ; IMPSOR ; IMPMTP ; IMPGRO ; IMPWHE ; IMPSUN ; IMPOTC</t>
+  </si>
+  <si>
+    <t>Output Activity Ratio</t>
+  </si>
+  <si>
+    <t>Crop yields</t>
+  </si>
+  <si>
+    <t>OutputActivityRatio</t>
+  </si>
+  <si>
+    <t>CRPMAI ; CRPCAN ; CRPGRO ; CRPMTP ; CRPOTC ; CRPPUL ; CRPSOR ; CRPWHE</t>
+  </si>
+  <si>
+    <t>Cost of public water supply distribution</t>
+  </si>
+  <si>
+    <t>DEMMINWAT ; DEMRESWAT ; DEMOTHWAT ; DEMPWRWAT ; DEMGOVWAT ; DEMAGRWAT</t>
+  </si>
+  <si>
+    <t>Cost of fuel distribution technologies</t>
+  </si>
+  <si>
+    <t>DEMINDELC ; DEMRESELC ; DEMCOMELC ; DEMAGRELC ; DEMTOURELC ; DEMTRAELC</t>
+  </si>
+  <si>
+    <t>User defined constraint</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total car capacity</t>
+  </si>
+  <si>
+    <t>UDCMultiplierTotalCapacity</t>
+  </si>
+  <si>
+    <t>TRAELCCARCUR ; TRAELCCARNEW</t>
+  </si>
+  <si>
+    <t>2TRACAREVCAP</t>
+  </si>
+  <si>
+    <t>TRAGSLCARCUR ; TRAGSLCARNEW ; TRADSLCARCUR ; TRADSLCARNEW; TRADSHCARNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total motorcycle capacity</t>
+  </si>
+  <si>
+    <t>TRAELCMCYCUR ; TRAELCMCYNEW</t>
+  </si>
+  <si>
+    <t>2TRAMCYEVCAP</t>
+  </si>
+  <si>
+    <t>TRAGSLMCYCUR ; TRAGSLMCYNEW ; TRADSLMCYNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total minibus capacity</t>
+  </si>
+  <si>
+    <t>TRAELCMNBCUR ; TRAELCMNBNEW</t>
+  </si>
+  <si>
+    <t>2TRAMNBEVCAP</t>
+  </si>
+  <si>
+    <t>TRAGSLMNBCUR ; TRAGSLMNBNEW ; TRADSLMNBCUR ; TRADSLMNBNEW; TRADSHMNBNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total bus capacity</t>
+  </si>
+  <si>
+    <t>TRAELCBUSCUR ; TRAELCBUSNEW</t>
+  </si>
+  <si>
+    <t>2TRABUSEVCAP</t>
+  </si>
+  <si>
+    <t>TRAGSLBUSCUR ; TRAGSLBUSNEW ; TRADSLBUSCUR ; TRADSLBUSNEW; TRADSHBUSNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total light truck capacity</t>
+  </si>
+  <si>
+    <t>TRAELCLTRCUR ; TRAELCLTRNEW</t>
+  </si>
+  <si>
+    <t>2TRALTREVCAP</t>
+  </si>
+  <si>
+    <t>TRAGSLLTRCUR ; TRAGSLLTRNEW ; TRADSLLTRCUR ; TRADSLLTRNEW; TRADSHLTRNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total medium truck capacity</t>
+  </si>
+  <si>
+    <t>TRAELCMTRCUR ; TRAELCMTRNEW</t>
+  </si>
+  <si>
+    <t>2TRAMTREVCAP</t>
+  </si>
+  <si>
+    <t>TRADSLMTRCUR ; TRADSLMTRNEW</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total heavy truck capacity</t>
+  </si>
+  <si>
+    <t>TRAELCHTRCUR ; TRAELCHTRNEW</t>
+  </si>
+  <si>
+    <t>2TRAHTREVCAP</t>
+  </si>
+  <si>
+    <t>TRADSLHTRCUR ; TRADSLHTRNEW</t>
+  </si>
+  <si>
+    <t>Forces water availability in 2050 to reduce to 75% of the 2020 value.</t>
+  </si>
+  <si>
+    <t>UDCConstant</t>
+  </si>
+  <si>
+    <t>RESTRICTWAT</t>
+  </si>
+  <si>
     <t>Collection rate</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum share of solid waste that should be collected </t>
   </si>
   <si>
-    <t>Scenario1</t>
-  </si>
-  <si>
-    <t>Time_Series</t>
-  </si>
-  <si>
-    <t>Final_Value</t>
-  </si>
-  <si>
     <t>UDCMultiplierActivity</t>
   </si>
   <si>
-    <t>NO</t>
-  </si>
-  <si>
     <t>WSTGEN</t>
   </si>
   <si>
     <t>COLWST</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Minimum share of liquid waste that should be collected </t>
   </si>
   <si>
@@ -231,217 +492,141 @@
     <t>COLLWT</t>
   </si>
   <si>
-    <t>Variable Costs</t>
-  </si>
-  <si>
-    <t>Variable Cost of crops technologies</t>
-  </si>
-  <si>
-    <t>VariableCost</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LNDPLAHR ; LNDPLALR ; LNDMAIHR ; LNDMAILR ; LNDCASHR ; LNDCASLR ; LNDBEAHR ; LNDBEALR ; LNDCOFHR ; LNDCOFLR ; LNDGROHR ; LNDGROLR ; LNDPTSHR ; LNDPTSLR ; LNDSUNHR ; LNDSUNLR ; LNDOTCHR ; LNDOTCLR ; LNDSORHR ; LNDSORLR ; LNDSESHR ; LNDSESLR ; LNDRICHR ; LNDRICHI ; LNDRICLR; LNDSOYHR ; LNDSOYLR ; LNDVEGHR ; LNDVEGLR
-</t>
-  </si>
-  <si>
-    <t>Fixed Costs</t>
-  </si>
-  <si>
-    <t>Fixed Cost of crops technologies</t>
-  </si>
-  <si>
-    <t>FixedCost</t>
-  </si>
-  <si>
-    <t>LNDPLAHR ; LNDPLALR ; LNDMAIHR ; LNDMAILR ; LNDCASHR ; LNDCASLR ; LNDBEAHR ; LNDBEALR ; LNDCOFHR ; LNDCOFLR ; LNDGROHR ; LNDGROLR ; LNDPTSHR ; LNDPTSLR ; LNDSUNHR ; LNDSUNLR ; LNDOTCHR ; LNDOTCLR ; LNDSORHR ; LNDSORLR ; LNDSESHR ; LNDSESLR ; LNDRICHR ; LNDRICHI ; LNDRICLR; LNDSOYHR ; LNDSOYLR ; LNDVEGHR ; LNDVEGLR</t>
-  </si>
-  <si>
-    <t>Capital Costs</t>
-  </si>
-  <si>
-    <t>Capital Cost of electric vehicles technologies</t>
-  </si>
-  <si>
-    <t>CapitalCost</t>
-  </si>
-  <si>
-    <t>TRAELCCARCUR ; TRAELCCARNEW ; TRAELCMCYCUR ; TRAELCMCYNEW ; TRAELCMNBCUR ; TRAELCMNBNEW ; TRAELCBUSCUR ; TRAELCBUSNEW ; TRAELCLTRCUR ; TRAELCLTRNEW ; TRAELCMTRCUR ; TRAELCMTRNEW ; TRAELCHTRCUR ; TRAELCHTRNEW</t>
-  </si>
-  <si>
-    <t>Fixed Cost of electric vehicles technologies</t>
-  </si>
-  <si>
-    <t>Capital Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>TRADSLCARCUR ; TRALPGCARNEW ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRALPGMNBNEW ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW ; TRALPGBUSNEW ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
-  </si>
-  <si>
-    <t>Fixed Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>Demand Growth</t>
-  </si>
-  <si>
-    <t>Changes in demand magnitude</t>
-  </si>
-  <si>
-    <t>AccumulatedAnnualDemand</t>
-  </si>
-  <si>
-    <t>RESLGTR ; RESLGTU ; RESCKNR ; RESCKNU ; RESSPHR ; RESWTHR ; RESWTHU ; RESCOLU ; RESELCOTHR ; RESELCOTHU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Import Cost of fuels </t>
-  </si>
-  <si>
-    <t>IMPDSL ; IMPGSL ; IMPKER ; IMPHFO ; IMPLPG</t>
-  </si>
-  <si>
-    <t>Input Activity Ratio</t>
-  </si>
-  <si>
-    <t>Activity ratio of inputs</t>
+    <t>Capital costs of utility-scale solar PV</t>
+  </si>
+  <si>
+    <t>PWRSOL001</t>
+  </si>
+  <si>
+    <t>CapacityFactor</t>
+  </si>
+  <si>
+    <t>Capital costs of the cement industry</t>
+  </si>
+  <si>
+    <t>DiscountRate</t>
+  </si>
+  <si>
+    <t>Reserve margin</t>
+  </si>
+  <si>
+    <t>PWRTRN</t>
+  </si>
+  <si>
+    <t>Demand growth in the agriculture sector</t>
+  </si>
+  <si>
+    <t>LVSSHP ; LVSGOA ; LVSOTH; CRPGRO; CRPMAI ; CRPMTP ; CRPPUL ; CRPOTC ; CRPSOR ; CRPSUN ; CRPWHE</t>
+  </si>
+  <si>
+    <t>Cattle population demand growth</t>
+  </si>
+  <si>
+    <t>LVSCTL</t>
+  </si>
+  <si>
+    <t>TotalAnnualMaxCapacity</t>
+  </si>
+  <si>
+    <t>Residual Capacity</t>
+  </si>
+  <si>
+    <t>Number_of_Runs</t>
+  </si>
+  <si>
+    <t>Scenario_to_Reproduce</t>
+  </si>
+  <si>
+    <t>Experiment_ID</t>
+  </si>
+  <si>
+    <t>Parallel_Use</t>
+  </si>
+  <si>
+    <t>Timeslices_model</t>
+  </si>
+  <si>
+    <t>Run_Base_Future</t>
+  </si>
+  <si>
+    <t>Run_RDM</t>
+  </si>
+  <si>
+    <t>Solver</t>
+  </si>
+  <si>
+    <t>OSeMOSYS_Model_Name</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Experiment</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>BWA</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>YearSplit</t>
+  </si>
+  <si>
+    <t>DiscountRateIdv</t>
+  </si>
+  <si>
+    <t>TradeRoute</t>
+  </si>
+  <si>
+    <t>DepreciationMethod</t>
+  </si>
+  <si>
+    <t>Conversionls</t>
+  </si>
+  <si>
+    <t>Conversionld</t>
+  </si>
+  <si>
+    <t>Conversionlh</t>
+  </si>
+  <si>
+    <t>DaySplit</t>
+  </si>
+  <si>
+    <t>DaysInDayType</t>
+  </si>
+  <si>
+    <t>SpecifiedAnnualDemand</t>
+  </si>
+  <si>
+    <t>SpecifiedDemandProfile</t>
+  </si>
+  <si>
+    <t>CapacityToActivityUnit</t>
+  </si>
+  <si>
+    <t>CapitalRecoveryFactor</t>
+  </si>
+  <si>
+    <t>CapacityOfOneTechnologyUnit</t>
+  </si>
+  <si>
+    <t>AvailabilityFactor</t>
+  </si>
+  <si>
+    <t>OperationalLife</t>
+  </si>
+  <si>
+    <t>ResidualCapacity</t>
   </si>
   <si>
     <t>InputActivityRatio</t>
   </si>
   <si>
-    <t xml:space="preserve"> INDOTHPLT ; INDMTRPLT ;  INDCHMPLT ; INDFBTPLT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INDOTHHTH ; INDOTHMDR ; INDELC ; INDMTRHTH ; INDMTRMDR ; INDELC ; INDCHMHTH ; INDCHMMDR ; INDELC ; INDFBTHTH ; INDELC ; INDFBTMDR </t>
-  </si>
-  <si>
-    <t>Capital Cost of Steel direct electric arc furnance with hydrogen, Capital Cost of cement industry kilns with CCS</t>
-  </si>
-  <si>
-    <t>INDIRSHDGDRI ; INDNGSKLNCCS ; INDBIOKLNCCS ; INDCOAKLNCCS</t>
-  </si>
-  <si>
-    <t>Capital Cost of Steel direct electric arc furnance with natural gas technologies , Capital Cost of cement industry kilns without CCS</t>
-  </si>
-  <si>
-    <t>INDIRSNGSDRI ; INDWSTKLN ; INDHFOKLN ; INDNGSKLN ; INDBIOKLN ; INDKLNCOA</t>
-  </si>
-  <si>
-    <t>Output Activity Ratio</t>
-  </si>
-  <si>
-    <t>Activity ratio of outputs</t>
-  </si>
-  <si>
-    <t>OutputActivityRatio</t>
-  </si>
-  <si>
-    <t>CRPPLA ; CRPMAI ; CRPCAS ; CRPBEA ; CRPCOF ; CRPGRO ; CRPPTS ; CRPSUN ; CRPOTC ; CRPSOR ; CRPSES ; CRPRIC ; CRPSOY ; CRPVEG</t>
-  </si>
-  <si>
-    <t>Number_of_Runs</t>
-  </si>
-  <si>
-    <t>Scenario_to_Reproduce</t>
-  </si>
-  <si>
-    <t>Experiment_ID</t>
-  </si>
-  <si>
-    <t>Parallel_Use</t>
-  </si>
-  <si>
-    <t>Timeslices_model</t>
-  </si>
-  <si>
-    <t>Run_Base_Future</t>
-  </si>
-  <si>
-    <t>Run_RDM</t>
-  </si>
-  <si>
-    <t>Solver</t>
-  </si>
-  <si>
-    <t>OSeMOSYS_Model_Name</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Experiment</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>glpk</t>
-  </si>
-  <si>
-    <t>model.v.5.3.txt</t>
-  </si>
-  <si>
-    <t>UGA</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>YearSplit</t>
-  </si>
-  <si>
-    <t>DiscountRate</t>
-  </si>
-  <si>
-    <t>DiscountRateIdv</t>
-  </si>
-  <si>
-    <t>TradeRoute</t>
-  </si>
-  <si>
-    <t>DepreciationMethod</t>
-  </si>
-  <si>
-    <t>Conversionls</t>
-  </si>
-  <si>
-    <t>Conversionld</t>
-  </si>
-  <si>
-    <t>Conversionlh</t>
-  </si>
-  <si>
-    <t>DaySplit</t>
-  </si>
-  <si>
-    <t>DaysInDayType</t>
-  </si>
-  <si>
-    <t>SpecifiedAnnualDemand</t>
-  </si>
-  <si>
-    <t>SpecifiedDemandProfile</t>
-  </si>
-  <si>
-    <t>CapacityToActivityUnit</t>
-  </si>
-  <si>
-    <t>CapitalRecoveryFactor</t>
-  </si>
-  <si>
-    <t>CapacityOfOneTechnologyUnit</t>
-  </si>
-  <si>
-    <t>CapacityFactor</t>
-  </si>
-  <si>
-    <t>AvailabilityFactor</t>
-  </si>
-  <si>
-    <t>OperationalLife</t>
-  </si>
-  <si>
-    <t>ResidualCapacity</t>
-  </si>
-  <si>
     <t>InputToNewCapacityRatio</t>
   </si>
   <si>
@@ -454,9 +639,6 @@
     <t>CapitalCostStorage</t>
   </si>
   <si>
-    <t>TotalAnnualMaxCapacity</t>
-  </si>
-  <si>
     <t>TotalAnnualMinCapacity</t>
   </si>
   <si>
@@ -523,15 +705,9 @@
     <t>TechnologyActivityByModeUpperLimit</t>
   </si>
   <si>
-    <t>UDCConstant</t>
-  </si>
-  <si>
     <t>UDCMultiplierNewCapacity</t>
   </si>
   <si>
-    <t>UDCMultiplierTotalCapacity</t>
-  </si>
-  <si>
     <t>UDCTag</t>
   </si>
   <si>
@@ -697,14 +873,35 @@
     <t>TotalDiscountedStorageCost</t>
   </si>
   <si>
-    <t>YES</t>
+    <t>RESMAR</t>
+  </si>
+  <si>
+    <t>Activity Limit</t>
+  </si>
+  <si>
+    <t>Electricity import availability</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>cplex</t>
+  </si>
+  <si>
+    <t>TRADSLCARCUR ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW  ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
+  </si>
+  <si>
+    <t>INDKILNBIOCCS; INDKILNCOACCS; INDKILNBIO; INDKILNCOA; INDKILNDSL; INDKILNLPG; INDKILNHFO; INDKILNCOA</t>
+  </si>
+  <si>
+    <t>model.v.5.4.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -721,13 +918,59 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -758,8 +1001,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -892,11 +1141,68 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -938,9 +1244,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -951,7 +1254,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -960,12 +1263,64 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF7575"/>
+      <color rgb="FFFF99FF"/>
+      <color rgb="FFFFA3A3"/>
+      <color rgb="FFFF0066"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1273,28 +1628,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:O53"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="15" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" style="15" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="15" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" style="15" customWidth="1"/>
     <col min="3" max="3" width="44" style="16" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" style="21" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" style="21" customWidth="1"/>
-    <col min="6" max="7" width="32.140625" style="21" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" style="21" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" style="21" customWidth="1"/>
-    <col min="10" max="10" width="54" style="21" customWidth="1"/>
-    <col min="11" max="11" width="79.7109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="49" style="22" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="45.85546875" style="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="44" style="22" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.85546875" style="20" customWidth="1"/>
-    <col min="16" max="16384" width="8.85546875" style="20"/>
+    <col min="4" max="4" width="24.44140625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" style="20" customWidth="1"/>
+    <col min="6" max="7" width="32.109375" style="20" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" style="20" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" style="20" customWidth="1"/>
+    <col min="10" max="10" width="54" style="15" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="79.6640625" style="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="49" style="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.88671875" style="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="44" style="21" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="15" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1325,7 +1681,7 @@
       <c r="J1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="39" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="18" t="s">
@@ -1341,7 +1697,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -1364,15 +1720,15 @@
         <v>2026</v>
       </c>
       <c r="H2" s="15">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I2" s="15">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="J2" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="40" t="s">
         <v>21</v>
       </c>
       <c r="L2" s="16" t="s">
@@ -1381,23 +1737,22 @@
       <c r="M2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="N2" s="15" t="s">
+      <c r="N2" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15">
-        <f t="shared" ref="A3:A15" si="0">1+A2</f>
         <v>2</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>17</v>
@@ -1412,40 +1767,39 @@
         <v>2026</v>
       </c>
       <c r="H3" s="15">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="I3" s="15">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="J3" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="40" t="s">
         <v>21</v>
       </c>
       <c r="L3" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O3" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>27</v>
-      </c>
-      <c r="M3" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O3" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="15">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>17</v>
@@ -1460,37 +1814,39 @@
         <v>2026</v>
       </c>
       <c r="H4" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="15">
-        <v>1.3</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="K4" t="s">
+        <v>1.5</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="23" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" s="16">
-        <v>1</v>
+      <c r="L4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>23</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" s="15" customFormat="1" ht="59.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15">
-        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>17</v>
@@ -1505,37 +1861,36 @@
         <v>2026</v>
       </c>
       <c r="H5" s="15">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I5" s="15">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="J5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" s="15" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="15">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>35</v>
-      </c>
-      <c r="K5" t="s">
-        <v>184</v>
-      </c>
-      <c r="L5" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="O5" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="15">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>38</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>17</v>
@@ -1550,40 +1905,39 @@
         <v>2026</v>
       </c>
       <c r="H6" s="15">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="I6" s="15">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="M6" s="15" t="s">
+      <c r="L6" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O6" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O6" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:15" s="15" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15">
-        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>17</v>
@@ -1598,40 +1952,39 @@
         <v>2026</v>
       </c>
       <c r="H7" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="15">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="K7" t="s">
+        <v>31</v>
+      </c>
+      <c r="K7" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="M7" s="15" t="s">
+      <c r="L7" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N7" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O7" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N7" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O7" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" s="15" customFormat="1" ht="112.15" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:15" s="15" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
-        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>17</v>
@@ -1646,40 +1999,39 @@
         <v>2026</v>
       </c>
       <c r="H8" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I8" s="15">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K8" t="s">
+        <v>36</v>
+      </c>
+      <c r="K8" s="40" t="s">
         <v>21</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="M8" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N8" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O8" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N8" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O8" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" s="15" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15">
-        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>17</v>
@@ -1694,40 +2046,39 @@
         <v>2026</v>
       </c>
       <c r="H9" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="15">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="J9" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="K9" t="s">
+        <v>1.5</v>
+      </c>
+      <c r="J9" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="M9" s="15" t="s">
+      <c r="M9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N9" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N9" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O9" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" s="15" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
-        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>17</v>
@@ -1742,40 +2093,39 @@
         <v>2026</v>
       </c>
       <c r="H10" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I10" s="15">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="K10" t="s">
+        <v>36</v>
+      </c>
+      <c r="K10" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="16" t="s">
-        <v>48</v>
-      </c>
-      <c r="M10" s="15" t="s">
+      <c r="L10" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O10" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N10" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="O10" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" s="19" customFormat="1" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
-        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>17</v>
@@ -1790,40 +2140,39 @@
         <v>2026</v>
       </c>
       <c r="H11" s="15">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="I11" s="15">
         <v>1.5</v>
       </c>
       <c r="J11" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="K11" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" s="40" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="M11" s="16">
-        <v>1</v>
-      </c>
-      <c r="N11" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N11" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O11" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="O11" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" s="19" customFormat="1" ht="61.9" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
-        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>17</v>
@@ -1838,40 +2187,39 @@
         <v>2026</v>
       </c>
       <c r="H12" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I12" s="15">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J12" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="K12" t="s">
+        <v>42</v>
+      </c>
+      <c r="K12" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L12" s="15" t="s">
-        <v>54</v>
+      <c r="L12" s="16" t="s">
+        <v>48</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="N12" s="15">
-        <v>1</v>
+        <v>23</v>
+      </c>
+      <c r="N12" s="16" t="s">
+        <v>23</v>
       </c>
       <c r="O12" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" s="19" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15">
-        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>17</v>
@@ -1886,40 +2234,39 @@
         <v>2026</v>
       </c>
       <c r="H13" s="15">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I13" s="15">
         <v>1.5</v>
       </c>
-      <c r="J13" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K13" t="s">
+      <c r="J13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" s="40" t="s">
         <v>21</v>
       </c>
       <c r="L13" s="16" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="M13" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N13" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O13" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N13" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="O13" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" s="19" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15">
-        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>17</v>
@@ -1934,40 +2281,39 @@
         <v>2026</v>
       </c>
       <c r="H14" s="15">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="I14" s="15">
-        <v>1.3</v>
-      </c>
-      <c r="J14" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" t="s">
+        <v>1.5</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="K14" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="16" t="s">
-        <v>59</v>
+      <c r="L14" s="22" t="s">
+        <v>43</v>
       </c>
       <c r="M14" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="N14" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O14" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="O14" s="16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15">
-        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>17</v>
@@ -1982,88 +2328,1276 @@
         <v>2026</v>
       </c>
       <c r="H15" s="15">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="I15" s="15">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J15" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="15">
+        <v>15</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H16" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I16" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J16" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="K16" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="O16" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="15">
+        <v>16</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H17" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I17" s="15">
+        <v>1</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K17" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L17" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="K15" t="s">
+      <c r="M17" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N17" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O17" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="15">
+        <v>17</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="33" t="s">
+        <v>60</v>
+      </c>
+      <c r="D18" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H18" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I18" s="32">
+        <v>1</v>
+      </c>
+      <c r="J18" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K18" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="23" t="s">
+      <c r="L18" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N18" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O18" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="15">
+        <v>18</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H19" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I19" s="15">
+        <v>1</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K19" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="M15" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="N15" s="15">
-        <v>1</v>
-      </c>
-      <c r="O15" s="16" t="s">
+      <c r="L19" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="N19" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O19" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="15">
+        <v>19</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E20" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H20" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I20" s="32">
+        <v>1</v>
+      </c>
+      <c r="J20" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K20" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L20" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="M20" s="33" t="s">
+        <v>67</v>
+      </c>
+      <c r="N20" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O20" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="15">
+        <v>20</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H21" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I21" s="15">
+        <v>1</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K21" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>71</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O21" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="15">
+        <v>21</v>
+      </c>
+      <c r="B22" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="33" t="s">
+        <v>69</v>
+      </c>
+      <c r="D22" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H22" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I22" s="32">
+        <v>1</v>
+      </c>
+      <c r="J22" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K22" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L22" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="M22" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="N22" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O22" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A23" s="15">
+        <v>22</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H23" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I23" s="15">
+        <v>1</v>
+      </c>
+      <c r="J23" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K23" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="N23" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O23" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" s="34" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="15">
+        <v>23</v>
+      </c>
+      <c r="B24" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="33" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H24" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I24" s="32">
+        <v>1</v>
+      </c>
+      <c r="J24" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K24" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L24" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="M24" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="N24" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O24" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="15">
+        <v>24</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H25" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I25" s="15">
+        <v>1</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K25" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L25" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="N25" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O25" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="15">
         <v>25</v>
       </c>
-    </row>
+      <c r="B26" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H26" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I26" s="32">
+        <v>1</v>
+      </c>
+      <c r="J26" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K26" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L26" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="M26" s="33" t="s">
+        <v>79</v>
+      </c>
+      <c r="N26" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O26" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="15">
+        <v>26</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H27" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I27" s="15">
+        <v>1</v>
+      </c>
+      <c r="J27" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K27" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L27" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="N27" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O27" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="15">
+        <v>27</v>
+      </c>
+      <c r="B28" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H28" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I28" s="32">
+        <v>1</v>
+      </c>
+      <c r="J28" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K28" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L28" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="M28" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="N28" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O28" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="15">
+        <v>28</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C29" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H29" s="15">
+        <v>0.93</v>
+      </c>
+      <c r="I29" s="15">
+        <v>1</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K29" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="L29" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="N29" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O29" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" s="34" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="15">
+        <v>29</v>
+      </c>
+      <c r="B30" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="D30" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="32">
+        <v>2026</v>
+      </c>
+      <c r="H30" s="32">
+        <v>0.93</v>
+      </c>
+      <c r="I30" s="32">
+        <v>1</v>
+      </c>
+      <c r="J30" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="K30" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L30" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="M30" s="33" t="s">
+        <v>87</v>
+      </c>
+      <c r="N30" s="33" t="s">
+        <v>23</v>
+      </c>
+      <c r="O30" s="33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="15">
+        <v>30</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H31" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I31" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="K31" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L31" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="M31" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N31" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O31" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" s="15" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="15">
+        <v>31</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="D32" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H32" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I32" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J32" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="K32" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="L32" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="M32" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="N32" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O32" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" s="15" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="15">
+        <v>32</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="31" t="s">
+        <v>18</v>
+      </c>
+      <c r="F33" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H33" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I33" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J33" s="28" t="s">
+        <v>94</v>
+      </c>
+      <c r="K33" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="L33" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="M33" s="29" t="s">
+        <v>99</v>
+      </c>
+      <c r="N33" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O33" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
+        <v>33</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H34" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I34" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J34" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="K34" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N34" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O34" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="15">
+        <v>34</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H35" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I35" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="K35" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N35" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O35" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="15">
+        <v>35</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H36" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I36" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="K36" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L36" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="M36" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="N36" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O36" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="15">
+        <v>36</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H37" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I37" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J37" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K37" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N37" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O37" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="15">
+        <v>37</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H38" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I38" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J38" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K38" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N38" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O38" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" s="38" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="15">
+        <v>38</v>
+      </c>
+      <c r="B39" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="C39" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="E39" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="36">
+        <v>2026</v>
+      </c>
+      <c r="H39" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="I39" s="36">
+        <v>1.5</v>
+      </c>
+      <c r="J39" s="36" t="s">
+        <v>111</v>
+      </c>
+      <c r="K39" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L39" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="M39" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="N39" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="O39" s="37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="15">
+        <v>39</v>
+      </c>
+      <c r="B40" s="32" t="s">
+        <v>228</v>
+      </c>
+      <c r="C40" s="33" t="s">
+        <v>229</v>
+      </c>
+      <c r="D40" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="E40" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="F40" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="32">
+        <v>2027</v>
+      </c>
+      <c r="H40" s="32">
+        <v>8</v>
+      </c>
+      <c r="I40" s="32">
+        <v>20</v>
+      </c>
+      <c r="J40" s="32" t="s">
+        <v>152</v>
+      </c>
+      <c r="K40" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L40" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="M40" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="N40" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="O40" s="37" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:N14" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:O40" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="UDCConstant"/>
+        <filter val="UDCMultiplierActivity"/>
+        <filter val="UDCMultiplierTotalCapacity"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EBD12E-40AD-42BC-9E38-C5D5CF6C4FA5}">
   <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>114</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>66</v>
+        <v>115</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>68</v>
+        <v>117</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>69</v>
+        <v>118</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>70</v>
+        <v>119</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>71</v>
+        <v>120</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="J1" s="26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+      <c r="J1" s="25" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>74</v>
+        <v>123</v>
       </c>
       <c r="C2" s="5">
         <v>1</v>
@@ -2075,19 +3609,19 @@
         <v>8</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>75</v>
+        <v>124</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>75</v>
+        <v>124</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>76</v>
+        <v>231</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="J2" s="25" t="s">
-        <v>78</v>
+        <v>234</v>
+      </c>
+      <c r="J2" s="24" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2096,249 +3630,249 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7095350F-2181-46D9-957F-C928CA3CEF59}">
   <dimension ref="A1:BG5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="21" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="23" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="22" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="18" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="23.109375" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="38" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="38.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="54" width="35.85546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="54" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="26" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="7.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>79</v>
+        <v>126</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>81</v>
+        <v>104</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>82</v>
+        <v>128</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>83</v>
+        <v>129</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>84</v>
+        <v>130</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>86</v>
+        <v>132</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="J1" t="s">
-        <v>88</v>
+        <v>134</v>
       </c>
       <c r="K1" t="s">
-        <v>89</v>
+        <v>135</v>
       </c>
       <c r="L1" t="s">
+        <v>136</v>
+      </c>
+      <c r="M1" t="s">
+        <v>137</v>
+      </c>
+      <c r="N1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>140</v>
+      </c>
+      <c r="R1" t="s">
+        <v>102</v>
+      </c>
+      <c r="S1" t="s">
+        <v>141</v>
+      </c>
+      <c r="T1" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="U1" t="s">
+        <v>143</v>
+      </c>
+      <c r="V1" t="s">
+        <v>144</v>
+      </c>
+      <c r="W1" t="s">
+        <v>145</v>
+      </c>
+      <c r="X1" t="s">
+        <v>146</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z1" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>156</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>157</v>
+      </c>
+      <c r="AO1" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AR1" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="AS1" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="AT1" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AV1" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>168</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>169</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>170</v>
+      </c>
+      <c r="BC1" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="M1" t="s">
-        <v>91</v>
-      </c>
-      <c r="N1" t="s">
-        <v>47</v>
-      </c>
-      <c r="O1" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q1" t="s">
+      <c r="BD1" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="R1" t="s">
-        <v>95</v>
-      </c>
-      <c r="S1" t="s">
-        <v>96</v>
-      </c>
-      <c r="T1" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="U1" t="s">
-        <v>98</v>
-      </c>
-      <c r="V1" t="s">
-        <v>53</v>
-      </c>
-      <c r="W1" t="s">
-        <v>99</v>
-      </c>
-      <c r="X1" t="s">
-        <v>100</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>62</v>
-      </c>
-      <c r="Z1" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>103</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>104</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>108</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>109</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>110</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>111</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>112</v>
-      </c>
-      <c r="AO1" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>115</v>
-      </c>
-      <c r="AR1" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="AS1" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="AT1" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>119</v>
-      </c>
-      <c r="AV1" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>102</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>121</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>122</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>123</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>124</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>125</v>
-      </c>
-      <c r="BC1" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="BD1" s="14" t="s">
-        <v>20</v>
-      </c>
       <c r="BE1" s="14" t="s">
-        <v>127</v>
+        <v>171</v>
       </c>
       <c r="BF1" s="14" t="s">
-        <v>128</v>
+        <v>61</v>
       </c>
       <c r="BG1" s="13" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" spans="1:59" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>173</v>
       </c>
       <c r="B2">
         <f t="shared" ref="B2:AQ2" si="0">+COUNTA(B3:B1048576)</f>
@@ -2573,183 +4107,183 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:59" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:59" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="J3" t="s">
-        <v>133</v>
+        <v>176</v>
       </c>
       <c r="K3" t="s">
-        <v>134</v>
+        <v>177</v>
       </c>
       <c r="L3" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="M3" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="N3" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="O3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="P3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="Q3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="R3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="S3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="T3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="U3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="V3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="W3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="X3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="Y3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="Z3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="AA3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AB3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AC3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AD3" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AE3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AF3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AG3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AH3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AI3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AJ3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AK3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AL3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AM3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AN3" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="AO3" s="13" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="AP3" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="AQ3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AR3" s="13" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AS3" s="13" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AT3" s="13" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AU3" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AV3" s="13" t="s">
-        <v>132</v>
+        <v>175</v>
       </c>
       <c r="AW3" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AX3" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AY3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="AZ3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BA3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BB3" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BC3" s="14" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BE3" s="14" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BF3" s="14" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="BG3" s="13" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="4" spans="1:59" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:59" x14ac:dyDescent="0.3">
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
@@ -2758,74 +4292,74 @@
       <c r="H4" s="13"/>
       <c r="I4" s="13"/>
       <c r="M4" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
       <c r="R4" t="s">
-        <v>131</v>
+        <v>174</v>
       </c>
       <c r="T4" s="13"/>
       <c r="V4" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="W4" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="X4" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="Y4" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
       <c r="Z4" s="13"/>
       <c r="AB4" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AM4" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="AO4" s="13"/>
       <c r="AQ4" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="AR4" s="13" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AS4" s="13" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AT4" s="13"/>
       <c r="AV4" s="13" t="s">
-        <v>137</v>
+        <v>180</v>
       </c>
       <c r="AY4" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AZ4" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="BA4" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="BB4" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="BC4" s="14"/>
       <c r="BD4" s="14" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="BE4" s="14" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="BF4" s="14" t="s">
-        <v>139</v>
+        <v>182</v>
       </c>
       <c r="BG4" s="13" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="5" spans="1:59" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59" x14ac:dyDescent="0.3">
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -2837,24 +4371,24 @@
       <c r="P5" s="13"/>
       <c r="T5" s="13"/>
       <c r="V5" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="Y5" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="Z5" s="13"/>
       <c r="AM5" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AO5" s="13"/>
       <c r="AQ5" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AR5" s="13" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AS5" s="13" t="s">
-        <v>140</v>
+        <v>183</v>
       </c>
       <c r="AT5" s="13"/>
       <c r="AV5" s="13"/>
@@ -2871,250 +4405,526 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C82A0652-0771-4DB6-84D0-EEBD0FFCEFAB}">
   <dimension ref="A1:B41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.44140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>141</v>
+        <v>184</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>187</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>146</v>
+        <v>189</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>191</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>149</v>
+        <v>192</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>150</v>
+        <v>193</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>154</v>
+        <v>197</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>204</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>162</v>
+        <v>205</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>180</v>
+        <v>223</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>183</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c4f98862-adfd-4d9c-a945-852f80f0eb51">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BAD73B84EC2FBA4AB6031CFB79C3D0E0" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d8e6320e34b5f71545ca20c1fb39b21">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c4f98862-adfd-4d9c-a945-852f80f0eb51" xmlns:ns3="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f42cd320e09c56919cd7e955403e252" ns2:_="" ns3:_="">
+    <xsd:import namespace="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
+    <xsd:import namespace="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c4f98862-adfd-4d9c-a945-852f80f0eb51" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="71f7bd95-1200-4052-9a4e-dfdf006e181b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="17" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="20" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6E40288-91D1-4CD6-86D1-178CC2AEE7EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAAAAB53-0ECA-470A-A9D1-4E2A413E8F82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED653E30-6791-4489-AE1B-B6DFD5392ED4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
+    <ds:schemaRef ds:uri="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Include new module to avoid infeasibilities related with EV UDC data
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,24 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A709DB37-B5A1-445B-B667-F0BF957A2960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDCDEDD-BAC6-4BD9-87EE-977459131693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{A38498C0-325E-4D75-9B65-6D8B75ECDFF0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Uncertainty_Table" sheetId="13" r:id="rId1"/>
-    <sheet name="Setup" sheetId="3" r:id="rId2"/>
-    <sheet name="Params_Sets_Vari" sheetId="14" r:id="rId3"/>
-    <sheet name="To_Print" sheetId="12" r:id="rId4"/>
+    <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
+    <sheet name="Setup" sheetId="2" r:id="rId2"/>
+    <sheet name="Params_Sets_Vari" sheetId="3" r:id="rId3"/>
+    <sheet name="To_Print" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$O$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$O$44</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -47,26 +44,17 @@
     <author>Climate Lead Group</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{2F50FA3F-EF55-4802-9EDB-FD7396EEA55E}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Options:
 - Linear: Performs a linear interpolation starting at the year of “Initial_Year_of_Uncertainty” and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
 - Constant: Performs a constant curve starting at the year of “Initial_Year_of_Uncertainty” with its value and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
@@ -76,76 +64,49 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{4B113B91-8C7D-4026-9B16-B744A1863E43}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the first set of InputActivityRatio is t: TECHNOLOGY, so you need to put sets of TECHNOLOGY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{56220757-0F04-471C-A32C-C1D985AB505F}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the second set of InputActivityRatio is f: COMODDITY so you need to put sets of COMODDITY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{8E8A5497-9CD0-462C-9F22-242368490FCA}">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the third set of InputActivityRatio is t: MODE_OF_OPERATION so you need to put sets of MODE_OF_OPERATION in this cell for that parameter.</t>
         </r>
@@ -161,26 +122,17 @@
     <author>Climate Lead Group</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{DBC5382B-8EB4-47E4-8B4B-119D1D2D7FE0}">
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Parameters paint in brown can not do a variation in RDM experiment.</t>
         </r>
       </text>
@@ -190,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="651" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="246">
   <si>
     <t>X_Num</t>
   </si>
@@ -276,7 +228,25 @@
     <t>Demand growth in the transport sector</t>
   </si>
   <si>
-    <t>TRACAR ; TRAMCY ; TRABUS ; TRAMNB ; TRALTR ; TRAMTR ; TRAHTR ; TRARAILF ; TRAAVI</t>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>TRABUS ; TRAMNB ; TRAMCY ; TRARAILF</t>
+  </si>
+  <si>
+    <t>UDCConstant</t>
+  </si>
+  <si>
+    <t>TRABUSACTCAP ; TRAMNBCAP ; TRAMCYCAP ; TRARAILFCAP</t>
+  </si>
+  <si>
+    <t>TRACAR</t>
+  </si>
+  <si>
+    <t>TRACARCAP</t>
+  </si>
+  <si>
+    <t>TRAMTR ; TRAHTR ; TRAAVI</t>
   </si>
   <si>
     <t>Capital Costs</t>
@@ -288,9 +258,6 @@
     <t>CapitalCost</t>
   </si>
   <si>
-    <t>YES</t>
-  </si>
-  <si>
     <t>TRAELCCARCUR ; TRAELCCARNEW ; TRAELCMCYCUR ; TRAELCMCYNEW ; TRAELCMNBCUR ; TRAELCMNBNEW ; TRAELCBUSCUR ; TRAELCBUSNEW ; TRAELCLTRCUR ; TRAELCLTRNEW ; TRAELCMTRCUR ; TRAELCMTRNEW ; TRAELCHTRCUR ; TRAELCHTRNEW</t>
   </si>
   <si>
@@ -312,6 +279,9 @@
     <t>Fixed Cost of ICE vehicles technologies</t>
   </si>
   <si>
+    <t>TRADSLCARCUR ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW  ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
+  </si>
+  <si>
     <t>Variable Costs</t>
   </si>
   <si>
@@ -462,9 +432,6 @@
     <t>Forces water availability in 2050 to reduce to 75% of the 2020 value.</t>
   </si>
   <si>
-    <t>UDCConstant</t>
-  </si>
-  <si>
     <t>RESTRICTWAT</t>
   </si>
   <si>
@@ -498,123 +465,168 @@
     <t>PWRSOL001</t>
   </si>
   <si>
+    <t>Capital costs of the cement industry</t>
+  </si>
+  <si>
+    <t>INDKILNBIOCCS ; INDKILNCOACCS ; INDKILNBIO ; INDKILNCOA ; INDKILNDSL ; INDKILNLPG ; INDKILNHFO ; INDKILNCOA</t>
+  </si>
+  <si>
+    <t>Reserve margin</t>
+  </si>
+  <si>
+    <t>PWRTRN</t>
+  </si>
+  <si>
+    <t>RESMAR</t>
+  </si>
+  <si>
+    <t>Demand growth in the agriculture sector</t>
+  </si>
+  <si>
+    <t>LVSSHP ; LVSGOA ; LVSOTH ; CRPGRO ; CRPMAI ; CRPMTP ; CRPPUL ; CRPOTC ; CRPSOR ; CRPSUN ; CRPWHE</t>
+  </si>
+  <si>
+    <t>Cattle population demand growth</t>
+  </si>
+  <si>
+    <t>LVSCTL</t>
+  </si>
+  <si>
+    <t>Residual Capacity</t>
+  </si>
+  <si>
+    <t>TotalAnnualMaxCapacity</t>
+  </si>
+  <si>
+    <t>Activity Limit</t>
+  </si>
+  <si>
+    <t>Electricity import availability</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>TotalTechnologyAnnualActivityUpperLimit</t>
+  </si>
+  <si>
+    <t>Number_of_Runs</t>
+  </si>
+  <si>
+    <t>Scenario_to_Reproduce</t>
+  </si>
+  <si>
+    <t>Experiment_ID</t>
+  </si>
+  <si>
+    <t>Parallel_Use</t>
+  </si>
+  <si>
+    <t>Timeslices_model</t>
+  </si>
+  <si>
+    <t>Run_Base_Future</t>
+  </si>
+  <si>
+    <t>Run_RDM</t>
+  </si>
+  <si>
+    <t>Solver</t>
+  </si>
+  <si>
+    <t>OSeMOSYS_Model_Name</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>EV_Conventional_Patterns</t>
+  </si>
+  <si>
+    <t>EV_Electric_Pattern</t>
+  </si>
+  <si>
+    <t>EV_UDCs</t>
+  </si>
+  <si>
+    <t>Experiment</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>cplex</t>
+  </si>
+  <si>
+    <t>model.v.5.4.txt</t>
+  </si>
+  <si>
+    <t>BWA</t>
+  </si>
+  <si>
+    <t>DSL;DSH;GSL</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>2TRACAREVCAP;2TRAMCYEVCAP;2TRABUSEVCAP;2TRAMNBEVCAP;2TRALTREVCAP;2TRAMTREVCAP;2TRAHTREVCAP</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>YearSplit</t>
+  </si>
+  <si>
+    <t>DiscountRate</t>
+  </si>
+  <si>
+    <t>DiscountRateIdv</t>
+  </si>
+  <si>
+    <t>TradeRoute</t>
+  </si>
+  <si>
+    <t>DepreciationMethod</t>
+  </si>
+  <si>
+    <t>Conversionls</t>
+  </si>
+  <si>
+    <t>Conversionld</t>
+  </si>
+  <si>
+    <t>Conversionlh</t>
+  </si>
+  <si>
+    <t>DaySplit</t>
+  </si>
+  <si>
+    <t>DaysInDayType</t>
+  </si>
+  <si>
+    <t>SpecifiedAnnualDemand</t>
+  </si>
+  <si>
+    <t>SpecifiedDemandProfile</t>
+  </si>
+  <si>
+    <t>CapacityToActivityUnit</t>
+  </si>
+  <si>
+    <t>CapitalRecoveryFactor</t>
+  </si>
+  <si>
+    <t>CapacityOfOneTechnologyUnit</t>
+  </si>
+  <si>
     <t>CapacityFactor</t>
   </si>
   <si>
-    <t>Capital costs of the cement industry</t>
-  </si>
-  <si>
-    <t>DiscountRate</t>
-  </si>
-  <si>
-    <t>Reserve margin</t>
-  </si>
-  <si>
-    <t>PWRTRN</t>
-  </si>
-  <si>
-    <t>Demand growth in the agriculture sector</t>
-  </si>
-  <si>
-    <t>LVSSHP ; LVSGOA ; LVSOTH; CRPGRO; CRPMAI ; CRPMTP ; CRPPUL ; CRPOTC ; CRPSOR ; CRPSUN ; CRPWHE</t>
-  </si>
-  <si>
-    <t>Cattle population demand growth</t>
-  </si>
-  <si>
-    <t>LVSCTL</t>
-  </si>
-  <si>
-    <t>TotalAnnualMaxCapacity</t>
-  </si>
-  <si>
-    <t>Residual Capacity</t>
-  </si>
-  <si>
-    <t>Number_of_Runs</t>
-  </si>
-  <si>
-    <t>Scenario_to_Reproduce</t>
-  </si>
-  <si>
-    <t>Experiment_ID</t>
-  </si>
-  <si>
-    <t>Parallel_Use</t>
-  </si>
-  <si>
-    <t>Timeslices_model</t>
-  </si>
-  <si>
-    <t>Run_Base_Future</t>
-  </si>
-  <si>
-    <t>Run_RDM</t>
-  </si>
-  <si>
-    <t>Solver</t>
-  </si>
-  <si>
-    <t>OSeMOSYS_Model_Name</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Experiment</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>BWA</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>YearSplit</t>
-  </si>
-  <si>
-    <t>DiscountRateIdv</t>
-  </si>
-  <si>
-    <t>TradeRoute</t>
-  </si>
-  <si>
-    <t>DepreciationMethod</t>
-  </si>
-  <si>
-    <t>Conversionls</t>
-  </si>
-  <si>
-    <t>Conversionld</t>
-  </si>
-  <si>
-    <t>Conversionlh</t>
-  </si>
-  <si>
-    <t>DaySplit</t>
-  </si>
-  <si>
-    <t>DaysInDayType</t>
-  </si>
-  <si>
-    <t>SpecifiedAnnualDemand</t>
-  </si>
-  <si>
-    <t>SpecifiedDemandProfile</t>
-  </si>
-  <si>
-    <t>CapacityToActivityUnit</t>
-  </si>
-  <si>
-    <t>CapitalRecoveryFactor</t>
-  </si>
-  <si>
-    <t>CapacityOfOneTechnologyUnit</t>
-  </si>
-  <si>
     <t>AvailabilityFactor</t>
   </si>
   <si>
@@ -648,9 +660,6 @@
     <t>TotalAnnualMinCapacityInvestment</t>
   </si>
   <si>
-    <t>TotalTechnologyAnnualActivityUpperLimit</t>
-  </si>
-  <si>
     <t>TotalTechnologyAnnualActivityLowerLimit</t>
   </si>
   <si>
@@ -871,37 +880,13 @@
   </si>
   <si>
     <t>TotalDiscountedStorageCost</t>
-  </si>
-  <si>
-    <t>RESMAR</t>
-  </si>
-  <si>
-    <t>Activity Limit</t>
-  </si>
-  <si>
-    <t>Electricity import availability</t>
-  </si>
-  <si>
-    <t>Step</t>
-  </si>
-  <si>
-    <t>cplex</t>
-  </si>
-  <si>
-    <t>TRADSLCARCUR ; TRADSLCARNEW ; TRADSLMCYNEW ; TRADSLMNBCUR ; TRADSLMNBNEW ; TRADSHMNBNEW ; TRADSLBUSCUR ; TRADSLBUSNEW  ; TRADSLBUSNEW ; TRADSLLTRCUR ; TRADSLLTRNEW ; TRADSHLTRNEW ; TRADSLMTRCUR ; TRADSLMTRNEW ; TRADSLHTRCUR ; TRADSLHTRNEW</t>
-  </si>
-  <si>
-    <t>INDKILNBIOCCS; INDKILNCOACCS; INDKILNBIO; INDKILNCOA; INDKILNDSL; INDKILNLPG; INDKILNHFO; INDKILNCOA</t>
-  </si>
-  <si>
-    <t>model.v.5.4.txt</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -913,25 +898,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1008,7 +974,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1141,68 +1107,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1244,7 +1153,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1254,7 +1162,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1263,49 +1171,47 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1313,14 +1219,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFFF7575"/>
-      <color rgb="FFFF99FF"/>
-      <color rgb="FFFFA3A3"/>
-      <color rgb="FFFF0066"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1628,29 +1526,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:O53"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O57"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" style="15" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" style="15" customWidth="1"/>
-    <col min="3" max="3" width="44" style="16" customWidth="1"/>
-    <col min="4" max="4" width="24.44140625" style="20" customWidth="1"/>
-    <col min="5" max="5" width="27.44140625" style="20" customWidth="1"/>
-    <col min="6" max="7" width="32.109375" style="20" customWidth="1"/>
-    <col min="8" max="8" width="13.5546875" style="20" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" style="20" customWidth="1"/>
-    <col min="10" max="10" width="54" style="15" customWidth="1"/>
-    <col min="11" max="11" width="14.5546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="79.6640625" style="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="49" style="21" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="45.88671875" style="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="44" style="21" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="19"/>
+    <col min="1" max="1" width="9.5546875" style="31" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" style="31" customWidth="1"/>
+    <col min="3" max="3" width="44" style="35" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" style="36" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" style="36" customWidth="1"/>
+    <col min="6" max="7" width="32.109375" style="36" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" style="36" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" style="36" customWidth="1"/>
+    <col min="10" max="10" width="54" style="31" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="79.6640625" style="35" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="49" style="37" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.88671875" style="36" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="44" style="37" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.88671875" style="32" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="15" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" s="31" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -1681,7 +1579,7 @@
       <c r="J1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="39" t="s">
+      <c r="K1" s="38" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="18" t="s">
@@ -1697,7 +1595,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -1728,7 +1626,7 @@
       <c r="J2" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="40" t="s">
+      <c r="K2" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L2" s="16" t="s">
@@ -1744,7 +1642,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15">
         <v>2</v>
       </c>
@@ -1775,7 +1673,7 @@
       <c r="J3" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="40" t="s">
+      <c r="K3" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L3" s="16" t="s">
@@ -1791,7 +1689,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15">
         <v>3</v>
       </c>
@@ -1822,11 +1720,11 @@
       <c r="J4" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K4" s="40" t="s">
-        <v>21</v>
+      <c r="K4" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M4" s="16" t="s">
         <v>23</v>
@@ -1838,15 +1736,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15">
         <v>4</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>17</v>
@@ -1867,30 +1765,33 @@
         <v>1.5</v>
       </c>
       <c r="J5" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="K5" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" s="23" t="s">
-        <v>33</v>
-      </c>
       <c r="M5" s="16" t="s">
         <v>23</v>
       </c>
       <c r="N5" s="16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" s="15" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="O5" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15">
         <v>5</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>17</v>
@@ -1911,13 +1812,13 @@
         <v>1.5</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="K6" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L6" s="23" t="s">
-        <v>33</v>
+        <v>20</v>
+      </c>
+      <c r="K6" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>32</v>
       </c>
       <c r="M6" s="16" t="s">
         <v>23</v>
@@ -1929,15 +1830,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:15" s="15" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15">
         <v>6</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>17</v>
@@ -1958,13 +1859,13 @@
         <v>1.5</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K7" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="K7" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L7" s="16" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="M7" s="16" t="s">
         <v>23</v>
@@ -1976,15 +1877,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="15" customFormat="1" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
         <v>7</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>17</v>
@@ -2005,13 +1906,13 @@
         <v>1.5</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="K8" s="40" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L8" s="16" t="s">
-        <v>232</v>
+        <v>34</v>
       </c>
       <c r="M8" s="16" t="s">
         <v>23</v>
@@ -2023,15 +1924,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15">
         <v>8</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>17</v>
@@ -2051,14 +1952,14 @@
       <c r="I9" s="15">
         <v>1.5</v>
       </c>
-      <c r="J9" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="K9" s="40" t="s">
+      <c r="J9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L9" s="22" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="M9" s="16" t="s">
         <v>23</v>
@@ -2066,19 +1967,17 @@
       <c r="N9" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
+      <c r="O9" s="20"/>
+    </row>
+    <row r="10" spans="1:15" s="31" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <v>9</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>17</v>
@@ -2099,13 +1998,13 @@
         <v>1.5</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="K10" s="40" t="s">
+        <v>41</v>
+      </c>
+      <c r="K10" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="M10" s="16" t="s">
         <v>23</v>
@@ -2117,15 +2016,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" s="31" customFormat="1" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>17</v>
@@ -2145,14 +2044,14 @@
       <c r="I11" s="15">
         <v>1.5</v>
       </c>
-      <c r="J11" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="K11" s="40" t="s">
+      <c r="J11" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K11" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="M11" s="16" t="s">
         <v>23</v>
@@ -2164,15 +2063,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" s="31" customFormat="1" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>17</v>
@@ -2192,14 +2091,14 @@
       <c r="I12" s="15">
         <v>1.5</v>
       </c>
-      <c r="J12" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="K12" s="40" t="s">
+      <c r="J12" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="M12" s="16" t="s">
         <v>23</v>
@@ -2211,15 +2110,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="15">
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>17</v>
@@ -2240,13 +2139,13 @@
         <v>1.5</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="K13" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="K13" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="16" t="s">
-        <v>50</v>
+      <c r="L13" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="M13" s="16" t="s">
         <v>23</v>
@@ -2258,15 +2157,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="15">
         <v>13</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>17</v>
@@ -2286,17 +2185,17 @@
       <c r="I14" s="15">
         <v>1.5</v>
       </c>
-      <c r="J14" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="K14" s="40" t="s">
+      <c r="J14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K14" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L14" s="22" t="s">
-        <v>43</v>
+      <c r="L14" s="21" t="s">
+        <v>49</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="N14" s="16" t="s">
         <v>23</v>
@@ -2305,15 +2204,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15">
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>17</v>
@@ -2334,29 +2233,33 @@
         <v>1.5</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="K15" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="K15" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="M15" s="16"/>
-      <c r="N15" s="16"/>
+        <v>52</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N15" s="16" t="s">
+        <v>23</v>
+      </c>
       <c r="O15" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="15">
         <v>15</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>17</v>
@@ -2377,27 +2280,33 @@
         <v>1.5</v>
       </c>
       <c r="J16" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="K16" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="K16" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L16" s="16" t="s">
-        <v>58</v>
+        <v>54</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N16" s="16" t="s">
+        <v>23</v>
       </c>
       <c r="O16" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15">
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>17</v>
@@ -2412,22 +2321,22 @@
         <v>2026</v>
       </c>
       <c r="H17" s="15">
-        <v>0.93</v>
+        <v>0.5</v>
       </c>
       <c r="I17" s="15">
-        <v>1</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K17" s="40" t="s">
-        <v>32</v>
+        <v>1.5</v>
+      </c>
+      <c r="J17" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="K17" s="25" t="s">
+        <v>21</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="N17" s="16" t="s">
         <v>23</v>
@@ -2436,62 +2345,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
         <v>17</v>
       </c>
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H18" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I18" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J18" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="K18" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M18" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H18" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I18" s="32">
-        <v>1</v>
-      </c>
-      <c r="J18" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K18" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L18" s="33" t="s">
-        <v>64</v>
-      </c>
-      <c r="M18" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="N18" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O18" s="33" t="s">
+      <c r="N18" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O18" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="15">
         <v>18</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>17</v>
@@ -2506,86 +2415,78 @@
         <v>2026</v>
       </c>
       <c r="H19" s="15">
-        <v>0.93</v>
+        <v>0.5</v>
       </c>
       <c r="I19" s="15">
-        <v>1</v>
-      </c>
-      <c r="J19" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K19" s="40" t="s">
-        <v>32</v>
+        <v>1.5</v>
+      </c>
+      <c r="J19" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="K19" s="25" t="s">
+        <v>21</v>
       </c>
       <c r="L19" s="16" t="s">
-        <v>66</v>
-      </c>
-      <c r="M19" s="16" t="s">
-        <v>67</v>
-      </c>
-      <c r="N19" s="16" t="s">
-        <v>23</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
       <c r="O19" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15">
         <v>19</v>
       </c>
-      <c r="B20" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" s="32" t="s">
+      <c r="B20" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E20" s="32" t="s">
+      <c r="E20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="32" t="s">
+      <c r="F20" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="32">
+      <c r="G20" s="15">
         <v>2026</v>
       </c>
-      <c r="H20" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I20" s="32">
-        <v>1</v>
-      </c>
-      <c r="J20" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K20" s="40" t="s">
+      <c r="H20" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I20" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J20" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="K20" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L20" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="M20" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="N20" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O20" s="33" t="s">
+      <c r="L20" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M20" s="20"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15">
         <v>20</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>17</v>
@@ -2606,16 +2507,16 @@
         <v>1</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K21" s="40" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="K21" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L21" s="16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="N21" s="16" t="s">
         <v>23</v>
@@ -2624,62 +2525,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="15">
         <v>21</v>
       </c>
-      <c r="B22" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="33" t="s">
+      <c r="B22" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="26">
+        <v>2026</v>
+      </c>
+      <c r="H22" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I22" s="26">
+        <v>1</v>
+      </c>
+      <c r="J22" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K22" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L22" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="M22" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="D22" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F22" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H22" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I22" s="32">
-        <v>1</v>
-      </c>
-      <c r="J22" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K22" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L22" s="33" t="s">
-        <v>72</v>
-      </c>
-      <c r="M22" s="33" t="s">
-        <v>71</v>
-      </c>
-      <c r="N22" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O22" s="33" t="s">
+      <c r="N22" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O22" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="15">
         <v>22</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>17</v>
@@ -2700,16 +2601,16 @@
         <v>1</v>
       </c>
       <c r="J23" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K23" s="40" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="K23" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L23" s="16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="N23" s="16" t="s">
         <v>23</v>
@@ -2718,62 +2619,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:15" s="34" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="15">
         <v>23</v>
       </c>
-      <c r="B24" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="33" t="s">
+      <c r="B24" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="26">
+        <v>2026</v>
+      </c>
+      <c r="H24" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I24" s="26">
+        <v>1</v>
+      </c>
+      <c r="J24" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K24" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L24" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="M24" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F24" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G24" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H24" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I24" s="32">
-        <v>1</v>
-      </c>
-      <c r="J24" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K24" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L24" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="M24" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="N24" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O24" s="33" t="s">
+      <c r="N24" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O24" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="15">
         <v>24</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C25" s="16" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>17</v>
@@ -2794,16 +2695,16 @@
         <v>1</v>
       </c>
       <c r="J25" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K25" s="40" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="K25" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L25" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="M25" s="16" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="N25" s="16" t="s">
         <v>23</v>
@@ -2812,62 +2713,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="15">
         <v>25</v>
       </c>
-      <c r="B26" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="33" t="s">
+      <c r="B26" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="26">
+        <v>2026</v>
+      </c>
+      <c r="H26" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I26" s="26">
+        <v>1</v>
+      </c>
+      <c r="J26" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K26" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L26" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="M26" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="D26" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E26" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G26" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H26" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I26" s="32">
-        <v>1</v>
-      </c>
-      <c r="J26" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K26" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L26" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="M26" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="N26" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O26" s="33" t="s">
+      <c r="N26" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O26" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15">
         <v>26</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C27" s="16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>17</v>
@@ -2888,16 +2789,16 @@
         <v>1</v>
       </c>
       <c r="J27" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K27" s="40" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="K27" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L27" s="16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="M27" s="16" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="N27" s="16" t="s">
         <v>23</v>
@@ -2906,62 +2807,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" s="33" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="15">
         <v>27</v>
       </c>
-      <c r="B28" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C28" s="33" t="s">
+      <c r="B28" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>79</v>
+      </c>
+      <c r="D28" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="26">
+        <v>2026</v>
+      </c>
+      <c r="H28" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I28" s="26">
+        <v>1</v>
+      </c>
+      <c r="J28" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K28" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L28" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="M28" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="D28" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E28" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G28" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H28" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I28" s="32">
-        <v>1</v>
-      </c>
-      <c r="J28" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K28" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L28" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="M28" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="N28" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O28" s="33" t="s">
+      <c r="N28" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O28" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="15">
         <v>28</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>17</v>
@@ -2982,16 +2883,16 @@
         <v>1</v>
       </c>
       <c r="J29" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K29" s="40" t="s">
-        <v>32</v>
+        <v>67</v>
+      </c>
+      <c r="K29" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L29" s="16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="N29" s="16" t="s">
         <v>23</v>
@@ -3000,62 +2901,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:15" s="34" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="15">
         <v>29</v>
       </c>
-      <c r="B30" s="32" t="s">
-        <v>59</v>
-      </c>
-      <c r="C30" s="33" t="s">
+      <c r="B30" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="26">
+        <v>2026</v>
+      </c>
+      <c r="H30" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I30" s="26">
+        <v>1</v>
+      </c>
+      <c r="J30" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K30" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L30" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="M30" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="D30" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F30" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="32">
-        <v>2026</v>
-      </c>
-      <c r="H30" s="32">
-        <v>0.93</v>
-      </c>
-      <c r="I30" s="32">
-        <v>1</v>
-      </c>
-      <c r="J30" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="K30" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="L30" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="M30" s="33" t="s">
-        <v>87</v>
-      </c>
-      <c r="N30" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="O30" s="33" t="s">
+      <c r="N30" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O30" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="15">
         <v>30</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>17</v>
@@ -3070,22 +2971,22 @@
         <v>2026</v>
       </c>
       <c r="H31" s="15">
-        <v>0.5</v>
+        <v>0.93</v>
       </c>
       <c r="I31" s="15">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="K31" s="40" t="s">
-        <v>21</v>
+        <v>67</v>
+      </c>
+      <c r="K31" s="25" t="s">
+        <v>28</v>
       </c>
       <c r="L31" s="16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="M31" s="16" t="s">
-        <v>23</v>
+        <v>89</v>
       </c>
       <c r="N31" s="16" t="s">
         <v>23</v>
@@ -3094,92 +2995,92 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:15" s="15" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15">
         <v>31</v>
       </c>
       <c r="B32" s="26" t="s">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="D32" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D32" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E32" s="30" t="s">
+      <c r="E32" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F32" s="30" t="s">
+      <c r="F32" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="26">
         <v>2026</v>
       </c>
-      <c r="H32" s="15">
-        <v>0.5</v>
-      </c>
-      <c r="I32" s="15">
-        <v>1.5</v>
+      <c r="H32" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I32" s="26">
+        <v>1</v>
       </c>
       <c r="J32" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="K32" s="41" t="s">
+        <v>67</v>
+      </c>
+      <c r="K32" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L32" s="27" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="M32" s="27" t="s">
-        <v>96</v>
-      </c>
-      <c r="N32" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="O32" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="N32" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O32" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:15" s="15" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15">
         <v>32</v>
       </c>
-      <c r="B33" s="28" t="s">
-        <v>92</v>
-      </c>
-      <c r="C33" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="D33" s="31" t="s">
+      <c r="B33" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E33" s="31" t="s">
+      <c r="E33" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F33" s="31" t="s">
+      <c r="F33" s="15" t="s">
         <v>19</v>
       </c>
       <c r="G33" s="15">
         <v>2026</v>
       </c>
       <c r="H33" s="15">
-        <v>0.5</v>
+        <v>0.93</v>
       </c>
       <c r="I33" s="15">
-        <v>1.5</v>
-      </c>
-      <c r="J33" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="K33" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="L33" s="29" t="s">
-        <v>98</v>
-      </c>
-      <c r="M33" s="29" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K33" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>93</v>
       </c>
       <c r="N33" s="16" t="s">
         <v>23</v>
@@ -3188,62 +3089,62 @@
         <v>24</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" s="33" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15">
         <v>33</v>
       </c>
-      <c r="B34" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="D34" s="15" t="s">
+      <c r="B34" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="D34" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="E34" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F34" s="15" t="s">
+      <c r="F34" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="G34" s="15">
+      <c r="G34" s="26">
         <v>2026</v>
       </c>
-      <c r="H34" s="15">
-        <v>0.5</v>
-      </c>
-      <c r="I34" s="15">
-        <v>1.5</v>
-      </c>
-      <c r="J34" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K34" s="40" t="s">
+      <c r="H34" s="26">
+        <v>0.93</v>
+      </c>
+      <c r="I34" s="26">
+        <v>1</v>
+      </c>
+      <c r="J34" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="K34" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L34" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="M34" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="N34" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="O34" s="16" t="s">
+      <c r="L34" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="M34" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="N34" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="O34" s="27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="15">
         <v>34</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="C35" s="16" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>17</v>
@@ -3264,13 +3165,13 @@
         <v>1.5</v>
       </c>
       <c r="J35" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="K35" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="K35" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L35" s="16" t="s">
-        <v>233</v>
+        <v>96</v>
       </c>
       <c r="M35" s="16" t="s">
         <v>23</v>
@@ -3282,23 +3183,23 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" s="31" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15">
         <v>35</v>
       </c>
-      <c r="B36" s="15" t="s">
-        <v>105</v>
-      </c>
-      <c r="C36" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="D36" s="15" t="s">
+      <c r="B36" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="C36" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="D36" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E36" s="15" t="s">
+      <c r="E36" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="15" t="s">
+      <c r="F36" s="25" t="s">
         <v>19</v>
       </c>
       <c r="G36" s="15">
@@ -3310,17 +3211,17 @@
       <c r="I36" s="15">
         <v>1.5</v>
       </c>
-      <c r="J36" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K36" s="40" t="s">
+      <c r="J36" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="K36" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L36" s="35" t="s">
-        <v>106</v>
-      </c>
-      <c r="M36" s="16" t="s">
-        <v>227</v>
+      <c r="L36" s="39" t="s">
+        <v>100</v>
+      </c>
+      <c r="M36" s="39" t="s">
+        <v>101</v>
       </c>
       <c r="N36" s="16" t="s">
         <v>23</v>
@@ -3329,23 +3230,23 @@
         <v>24</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" s="31" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="15">
         <v>36</v>
       </c>
-      <c r="B37" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C37" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="D37" s="15" t="s">
+      <c r="B37" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="C37" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="D37" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="E37" s="15" t="s">
+      <c r="E37" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="F37" s="15" t="s">
+      <c r="F37" s="25" t="s">
         <v>19</v>
       </c>
       <c r="G37" s="15">
@@ -3357,17 +3258,17 @@
       <c r="I37" s="15">
         <v>1.5</v>
       </c>
-      <c r="J37" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="K37" s="40" t="s">
+      <c r="J37" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="K37" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L37" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="M37" s="16" t="s">
-        <v>23</v>
+      <c r="L37" s="39" t="s">
+        <v>103</v>
+      </c>
+      <c r="M37" s="39" t="s">
+        <v>104</v>
       </c>
       <c r="N37" s="16" t="s">
         <v>23</v>
@@ -3376,15 +3277,15 @@
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="15">
         <v>37</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D38" s="15" t="s">
         <v>17</v>
@@ -3405,13 +3306,13 @@
         <v>1.5</v>
       </c>
       <c r="J38" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="K38" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="K38" s="25" t="s">
         <v>21</v>
       </c>
       <c r="L38" s="16" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="M38" s="16" t="s">
         <v>23</v>
@@ -3423,133 +3324,312 @@
         <v>24</v>
       </c>
     </row>
-    <row r="39" spans="1:15" s="38" customFormat="1" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="15">
         <v>38</v>
       </c>
-      <c r="B39" s="36" t="s">
-        <v>112</v>
-      </c>
-      <c r="C39" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="D39" s="36" t="s">
+      <c r="B39" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="36" t="s">
+      <c r="E39" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="F39" s="36" t="s">
+      <c r="F39" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G39" s="36">
+      <c r="G39" s="15">
         <v>2026</v>
       </c>
-      <c r="H39" s="36">
+      <c r="H39" s="15">
         <v>0.5</v>
       </c>
-      <c r="I39" s="36">
+      <c r="I39" s="15">
         <v>1.5</v>
       </c>
-      <c r="J39" s="36" t="s">
-        <v>111</v>
-      </c>
-      <c r="K39" s="40" t="s">
+      <c r="J39" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="K39" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L39" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="M39" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="N39" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="O39" s="37" t="s">
+      <c r="L39" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N39" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O39" s="16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="40" spans="1:15" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="15">
         <v>39</v>
       </c>
-      <c r="B40" s="32" t="s">
-        <v>228</v>
-      </c>
-      <c r="C40" s="33" t="s">
-        <v>229</v>
-      </c>
-      <c r="D40" s="32" t="s">
+      <c r="B40" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E40" s="32" t="s">
-        <v>230</v>
-      </c>
-      <c r="F40" s="32" t="s">
+      <c r="E40" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G40" s="32">
+      <c r="G40" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H40" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I40" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="K40" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L40" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="N40" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O40" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="15">
+        <v>40</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H41" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I41" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J41" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K41" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N41" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O41" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="15">
+        <v>41</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C42" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G42" s="15">
+        <v>2026</v>
+      </c>
+      <c r="H42" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="I42" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="K42" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L42" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N42" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O42" s="16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" s="34" customFormat="1" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="15">
+        <v>42</v>
+      </c>
+      <c r="B43" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="D43" s="29" t="s">
+        <v>17</v>
+      </c>
+      <c r="E43" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="F43" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="G43" s="29">
+        <v>2026</v>
+      </c>
+      <c r="H43" s="29">
+        <v>0.5</v>
+      </c>
+      <c r="I43" s="29">
+        <v>1.5</v>
+      </c>
+      <c r="J43" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="K43" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="L43" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="M43" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="N43" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="O43" s="30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="15">
+        <v>43</v>
+      </c>
+      <c r="B44" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="D44" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="E44" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="F44" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G44" s="26">
         <v>2027</v>
       </c>
-      <c r="H40" s="32">
+      <c r="H44" s="26">
         <v>8</v>
       </c>
-      <c r="I40" s="32">
+      <c r="I44" s="26">
         <v>20</v>
       </c>
-      <c r="J40" s="32" t="s">
-        <v>152</v>
-      </c>
-      <c r="K40" s="40" t="s">
+      <c r="J44" s="26" t="s">
+        <v>121</v>
+      </c>
+      <c r="K44" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="L40" s="33" t="s">
-        <v>48</v>
-      </c>
-      <c r="M40" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="N40" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="O40" s="37" t="s">
+      <c r="L44" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="M44" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="N44" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="O44" s="30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="41" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:15" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <autoFilter ref="A1:O40" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="UDCConstant"/>
-        <filter val="UDCMultiplierActivity"/>
-        <filter val="UDCMultiplierTotalCapacity"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <autoFilter ref="A1:O44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8EBD12E-40AD-42BC-9E38-C5D5CF6C4FA5}">
-  <dimension ref="A1:J2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -3558,46 +3638,56 @@
     <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="J1" s="25" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="L1" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="M1" s="24" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="C2" s="5">
         <v>1</v>
@@ -3609,19 +3699,28 @@
         <v>8</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>231</v>
+        <v>138</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="J2" s="24" t="s">
-        <v>125</v>
+        <v>139</v>
+      </c>
+      <c r="J2" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="K2" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="L2" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="M2" s="40" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -3630,7 +3729,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7095350F-2181-46D9-957F-C928CA3CEF59}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:BG5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3693,186 +3792,186 @@
   <sheetData>
     <row r="1" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="B1" t="s">
-        <v>127</v>
+        <v>145</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>104</v>
+        <v>146</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>133</v>
+        <v>152</v>
       </c>
       <c r="J1" t="s">
-        <v>134</v>
+        <v>153</v>
       </c>
       <c r="K1" t="s">
-        <v>135</v>
+        <v>154</v>
       </c>
       <c r="L1" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="M1" t="s">
-        <v>137</v>
+        <v>156</v>
       </c>
       <c r="N1" t="s">
         <v>20</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="Q1" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="R1" t="s">
-        <v>102</v>
+        <v>160</v>
       </c>
       <c r="S1" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="T1" s="13" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="U1" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="V1" t="s">
-        <v>144</v>
+        <v>164</v>
       </c>
       <c r="W1" t="s">
-        <v>145</v>
+        <v>165</v>
       </c>
       <c r="X1" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="Y1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="Z1" s="13" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="AA1" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="AB1" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="AC1" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="AD1" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="AE1" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="AF1" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="AG1" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="AH1" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="AI1" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="AJ1" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="AK1" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="AL1" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="AM1" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="AN1" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="AO1" s="13" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="AP1" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="AQ1" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="AR1" s="13" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="AS1" s="13" t="s">
-        <v>162</v>
+        <v>181</v>
       </c>
       <c r="AT1" s="13" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="AU1" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="AV1" s="13" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="AW1" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="AX1" t="s">
-        <v>166</v>
+        <v>185</v>
       </c>
       <c r="AY1" t="s">
-        <v>167</v>
+        <v>186</v>
       </c>
       <c r="AZ1" t="s">
-        <v>168</v>
+        <v>187</v>
       </c>
       <c r="BA1" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="BB1" t="s">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="BC1" s="14" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="BD1" s="14" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="BE1" s="14" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="BF1" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="BG1" s="13" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="B2">
         <f t="shared" ref="B2:AQ2" si="0">+COUNTA(B3:B1048576)</f>
@@ -4109,178 +4208,178 @@
     </row>
     <row r="3" spans="1:59" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="J3" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K3" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="L3" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="M3" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="N3" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="O3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="P3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="Q3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="R3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="S3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="T3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="U3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="V3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="W3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="X3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="Y3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="Z3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="AA3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AB3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AC3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AD3" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AE3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AF3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AG3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AH3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AI3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AJ3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AK3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AL3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AM3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AN3" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="AO3" s="13" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="AP3" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="AQ3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AR3" s="13" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AS3" s="13" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AT3" s="13" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AU3" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AV3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="AW3" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AX3" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AY3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="AZ3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BA3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BB3" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BC3" s="14" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BE3" s="14" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BF3" s="14" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="BG3" s="13" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:59" x14ac:dyDescent="0.3">
@@ -4292,71 +4391,71 @@
       <c r="H4" s="13"/>
       <c r="I4" s="13"/>
       <c r="M4" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
       <c r="R4" t="s">
-        <v>174</v>
+        <v>193</v>
       </c>
       <c r="T4" s="13"/>
       <c r="V4" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="W4" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="X4" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="Y4" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="Z4" s="13"/>
       <c r="AB4" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AM4" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="AO4" s="13"/>
       <c r="AQ4" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="AR4" s="13" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AS4" s="13" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AT4" s="13"/>
       <c r="AV4" s="13" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="AY4" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AZ4" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="BA4" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="BB4" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="BC4" s="14"/>
       <c r="BD4" s="14" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="BE4" s="14" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="BF4" s="14" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="BG4" s="13" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
     </row>
     <row r="5" spans="1:59" x14ac:dyDescent="0.3">
@@ -4371,24 +4470,24 @@
       <c r="P5" s="13"/>
       <c r="T5" s="13"/>
       <c r="V5" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="Y5" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="Z5" s="13"/>
       <c r="AM5" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AO5" s="13"/>
       <c r="AQ5" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AR5" s="13" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AS5" s="13" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="AT5" s="13"/>
       <c r="AV5" s="13"/>
@@ -4405,7 +4504,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C82A0652-0771-4DB6-84D0-EEBD0FFCEFAB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4415,516 +4514,243 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>189</v>
+        <v>208</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>190</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>195</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>198</v>
+        <v>217</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>205</v>
+        <v>224</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>206</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>210</v>
+        <v>229</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>212</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>213</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>215</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>218</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>219</v>
+        <v>238</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>222</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>223</v>
+        <v>242</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>224</v>
+        <v>243</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>225</v>
+        <v>244</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>226</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c4f98862-adfd-4d9c-a945-852f80f0eb51">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BAD73B84EC2FBA4AB6031CFB79C3D0E0" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1d8e6320e34b5f71545ca20c1fb39b21">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c4f98862-adfd-4d9c-a945-852f80f0eb51" xmlns:ns3="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f42cd320e09c56919cd7e955403e252" ns2:_="" ns3:_="">
-    <xsd:import namespace="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
-    <xsd:import namespace="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c4f98862-adfd-4d9c-a945-852f80f0eb51" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="71f7bd95-1200-4052-9a4e-dfdf006e181b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="14" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="17" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="20" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6E40288-91D1-4CD6-86D1-178CC2AEE7EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAAAAB53-0ECA-470A-A9D1-4E2A413E8F82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED653E30-6791-4489-AE1B-B6DFD5392ED4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c4f98862-adfd-4d9c-a945-852f80f0eb51"/>
-    <ds:schemaRef ds:uri="b9355cc9-2d41-4aa9-bfbc-bd016a1e1a01"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updated OAR in interface table
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RDM\github_RDM\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86749A2B-E8B2-4231-B153-393D9055C9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8BB833C-281A-4BAF-8531-3EF6D31DBAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -142,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="199">
   <si>
     <t>X_Num</t>
   </si>
@@ -732,13 +732,13 @@
     <t>Demand growth in the buildings sector</t>
   </si>
   <si>
+    <t>Fixed Costs</t>
+  </si>
+  <si>
+    <t>Fixed Cost of electric vehicles technologies</t>
+  </si>
+  <si>
     <t>RESCKN ; RESLGT ; RESCOL ; RESWHT ; RESHEL ; RESELCOTH ; COMELCOTH ; COMHET ; TOURELCOTH ; TOURHET</t>
-  </si>
-  <si>
-    <t>Fixed Costs</t>
-  </si>
-  <si>
-    <t>Fixed Cost of electric vehicles technologies</t>
   </si>
 </sst>
 </file>
@@ -998,7 +998,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1039,9 +1039,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1418,23 +1415,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" style="3" customWidth="1"/>
     <col min="2" max="2" width="28.28515625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="44" style="30" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" style="31" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" style="31" customWidth="1"/>
-    <col min="6" max="7" width="32.140625" style="31" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" style="31" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" style="31" customWidth="1"/>
+    <col min="3" max="3" width="44" style="29" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" style="30" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" style="30" customWidth="1"/>
+    <col min="6" max="7" width="32.140625" style="30" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="30" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" style="30" customWidth="1"/>
     <col min="10" max="10" width="54" style="3" customWidth="1"/>
     <col min="11" max="11" width="14.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="79.7109375" style="30" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="49" style="32" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="45.85546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="44" style="32" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="81.5703125" style="29" customWidth="1"/>
+    <col min="13" max="13" width="49" style="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.85546875" style="30" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="44" style="31" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1469,7 +1466,7 @@
       <c r="J1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="33" t="s">
+      <c r="K1" s="32" t="s">
         <v>10</v>
       </c>
       <c r="L1" s="18" t="s">
@@ -1516,11 +1513,11 @@
       <c r="J2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="K2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L2" s="22" t="s">
-        <v>196</v>
+      <c r="L2" s="21" t="s">
+        <v>198</v>
       </c>
       <c r="M2" s="16" t="s">
         <v>20</v>
@@ -1528,7 +1525,7 @@
       <c r="N2" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="O2" s="19" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1563,10 +1560,10 @@
       <c r="J3" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="K3" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="22" t="s">
+      <c r="L3" s="21" t="s">
         <v>27</v>
       </c>
       <c r="M3" s="16" t="s">
@@ -1575,52 +1572,52 @@
       <c r="N3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="O3" s="20"/>
-    </row>
-    <row r="4" spans="1:15" s="37" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="O3" s="19"/>
+    </row>
+    <row r="4" spans="1:15" s="36" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="17">
         <v>3</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="36" t="s">
+        <v>196</v>
+      </c>
+      <c r="C4" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="C4" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="37" t="s">
+      <c r="E4" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="37">
+      <c r="G4" s="36">
         <v>2026</v>
       </c>
-      <c r="H4" s="37">
+      <c r="H4" s="36">
         <v>0.5</v>
       </c>
-      <c r="I4" s="37">
+      <c r="I4" s="36">
         <v>1.5</v>
       </c>
-      <c r="J4" s="37" t="s">
+      <c r="J4" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="39" t="s">
+      <c r="K4" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="L4" s="40" t="s">
+      <c r="L4" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="M4" s="38" t="s">
+      <c r="M4" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="N4" s="38" t="s">
+      <c r="N4" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="38" t="s">
+      <c r="O4" s="37" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1655,7 +1652,7 @@
       <c r="J5" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="K5" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L5" s="16" t="s">
@@ -1702,10 +1699,10 @@
       <c r="J6" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K6" s="25" t="s">
+      <c r="K6" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="L6" s="20" t="s">
         <v>34</v>
       </c>
       <c r="M6" s="16" t="s">
@@ -1749,7 +1746,7 @@
       <c r="J7" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="25" t="s">
+      <c r="K7" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L7" s="16" t="s">
@@ -1765,7 +1762,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:15" s="36" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" s="35" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="17">
         <v>7</v>
       </c>
@@ -1796,7 +1793,7 @@
       <c r="J8" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K8" s="35" t="s">
+      <c r="K8" s="34" t="s">
         <v>19</v>
       </c>
       <c r="L8" s="16" t="s">
@@ -1843,7 +1840,7 @@
       <c r="J9" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K9" s="25" t="s">
+      <c r="K9" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L9" s="16" t="s">
@@ -1890,7 +1887,7 @@
       <c r="J10" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="K10" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L10" s="16" t="s">
@@ -1937,17 +1934,17 @@
       <c r="J11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="21" t="s">
+      <c r="L11" s="20" t="s">
         <v>34</v>
       </c>
       <c r="M11" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="N11" s="16" t="s">
-        <v>20</v>
+      <c r="N11" s="16">
+        <v>1</v>
       </c>
       <c r="O11" s="16" t="s">
         <v>21</v>
@@ -1984,14 +1981,18 @@
       <c r="J12" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="K12" s="25" t="s">
+      <c r="K12" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L12" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="M12" s="20"/>
-      <c r="N12" s="19"/>
+      <c r="M12" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="N12" s="16" t="s">
+        <v>20</v>
+      </c>
       <c r="O12" s="16" t="s">
         <v>21</v>
       </c>
@@ -2027,7 +2028,7 @@
       <c r="J13" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K13" s="25" t="s">
+      <c r="K13" s="24" t="s">
         <v>22</v>
       </c>
       <c r="L13" s="16" t="s">
@@ -2047,46 +2048,46 @@
       <c r="A14" s="17">
         <v>13</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="25">
         <v>2026</v>
       </c>
-      <c r="H14" s="26">
+      <c r="H14" s="25">
         <v>0.93</v>
       </c>
-      <c r="I14" s="26">
-        <v>1</v>
-      </c>
-      <c r="J14" s="26" t="s">
+      <c r="I14" s="25">
+        <v>1</v>
+      </c>
+      <c r="J14" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="K14" s="25" t="s">
+      <c r="K14" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L14" s="27" t="s">
+      <c r="L14" s="26" t="s">
         <v>52</v>
       </c>
       <c r="M14" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="N14" s="27" t="s">
+      <c r="N14" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="O14" s="27" t="s">
+      <c r="O14" s="26" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2121,7 +2122,7 @@
       <c r="J15" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="K15" s="25" t="s">
+      <c r="K15" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L15" s="16" t="s">
@@ -2137,7 +2138,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:15" s="36" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" s="35" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="17">
         <v>15</v>
       </c>
@@ -2168,7 +2169,7 @@
       <c r="J16" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K16" s="35" t="s">
+      <c r="K16" s="34" t="s">
         <v>19</v>
       </c>
       <c r="L16" s="16" t="s">
@@ -2215,7 +2216,7 @@
       <c r="J17" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="K17" s="25" t="s">
+      <c r="K17" s="24" t="s">
         <v>19</v>
       </c>
       <c r="L17" s="16" t="s">
@@ -2262,10 +2263,10 @@
       <c r="J18" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="K18" s="25" t="s">
+      <c r="K18" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L18" s="28" t="s">
+      <c r="L18" s="27" t="s">
         <v>59</v>
       </c>
       <c r="M18" s="16" t="s">
@@ -2282,46 +2283,46 @@
       <c r="A19" s="17">
         <v>18</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="B19" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="27" t="s">
+      <c r="C19" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="F19" s="26" t="s">
+      <c r="F19" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="26">
+      <c r="G19" s="25">
         <v>2027</v>
       </c>
-      <c r="H19" s="26">
+      <c r="H19" s="25">
         <v>8</v>
       </c>
-      <c r="I19" s="26">
+      <c r="I19" s="25">
         <v>20</v>
       </c>
-      <c r="J19" s="26" t="s">
+      <c r="J19" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="K19" s="25" t="s">
+      <c r="K19" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="L19" s="27" t="s">
+      <c r="L19" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="M19" s="29" t="s">
+      <c r="M19" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="N19" s="29" t="s">
+      <c r="N19" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="O19" s="29" t="s">
+      <c r="O19" s="28" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2337,7 +2338,6 @@
     <row r="29" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:O19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2388,16 +2388,16 @@
       <c r="I1" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="K1" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="L1" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="23" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2429,16 +2429,16 @@
       <c r="I2" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" s="22" t="s">
         <v>84</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="L2" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="M2" s="34" t="s">
+      <c r="M2" s="33" t="s">
         <v>86</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add configurable solver threads and CBC time limit from Setup sheet
Add Threads_CPLEX_Gurobi and Time_CBC columns to the Setup sheet to
configure CPLEX/Gurobi thread count and CBC time limit from the Excel
interface, replacing the previously hardcoded values.
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -8,18 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ClimateLeadGroup\Desktop\CLG_repositories\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22C06AD2-3EE9-4707-AE76-2D55DCED6D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08DB8E74-68FF-4825-9D7A-79CC27EC08AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Uncertainty_Table" sheetId="6" r:id="rId1"/>
+    <sheet name="Uncertainty_Table" sheetId="1" r:id="rId1"/>
     <sheet name="Setup" sheetId="2" r:id="rId2"/>
     <sheet name="Params_Sets_Vari" sheetId="3" r:id="rId3"/>
     <sheet name="To_Print" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$O$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Uncertainty_Table!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,26 +44,17 @@
     <author>Climate Lead Group</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{F6C5D05F-274C-49C6-900D-09B08523D85C}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Options:
 - Linear: Performs a linear interpolation starting at the year of “Initial_Year_of_Uncertainty” and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
 - Constant: Performs a constant curve starting at the year of “Initial_Year_of_Uncertainty” with its value and ending at the last year of the model. (The value of the “Explored_Parameter_of_X” must be “Final_value”).
@@ -73,76 +64,49 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{E07CD746-DD45-4131-9451-DBCEB738338E}">
+    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the first set of InputActivityRatio is t: TECHNOLOGY, so you need to put sets of TECHNOLOGY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{02D7225D-0569-4C60-8C94-C7232840BA6A}">
+    <comment ref="M1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the second set of InputActivityRatio is f: COMODDITY so you need to put sets of COMODDITY in this cell for that parameter.</t>
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{F371F3CF-DDBB-4153-8933-AC6411724897}">
+    <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
       <text>
         <r>
           <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
+            <scheme val="minor"/>
           </rPr>
-          <t>Climate Lead Group:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
+          <t>Climate Lead Group:
 Check "Params_Sets_Vari" for each parameter involved. You need put sets related with the parameter in the same order as you see in the sheet.
 Fo example the third set of InputActivityRatio is t: MODE_OF_OPERATION so you need to put sets of MODE_OF_OPERATION in this cell for that parameter.</t>
         </r>
@@ -178,7 +142,76 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="214">
+  <si>
+    <t>Number_of_Runs</t>
+  </si>
+  <si>
+    <t>Scenario_to_Reproduce</t>
+  </si>
+  <si>
+    <t>Experiment_ID</t>
+  </si>
+  <si>
+    <t>Parallel_Use</t>
+  </si>
+  <si>
+    <t>Timeslices_model</t>
+  </si>
+  <si>
+    <t>Run_Base_Future</t>
+  </si>
+  <si>
+    <t>Run_RDM</t>
+  </si>
+  <si>
+    <t>Solver</t>
+  </si>
+  <si>
+    <t>OSeMOSYS_Model_Name</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>EV_Conventional_Patterns</t>
+  </si>
+  <si>
+    <t>EV_Electric_Pattern</t>
+  </si>
+  <si>
+    <t>EV_UDCs</t>
+  </si>
+  <si>
+    <t>Threads_CPLEX_Gurobi</t>
+  </si>
+  <si>
+    <t>Time_CBC</t>
+  </si>
+  <si>
+    <t>Experiment</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>cplex</t>
+  </si>
+  <si>
+    <t>model.v.5.4.txt</t>
+  </si>
+  <si>
+    <t>BWA</t>
+  </si>
+  <si>
+    <t>DSL;DSH;GSL</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>2TRACAREVCAP;2TRAMCYEVCAP;2TRABUSEVCAP;2TRAMNBEVCAP;2TRALTREVCAP;2TRAMTREVCAP;2TRAHTREVCAP</t>
+  </si>
   <si>
     <t>X_Num</t>
   </si>
@@ -228,6 +261,9 @@
     <t>Demand Growth</t>
   </si>
   <si>
+    <t>Demand growth in the buildings, industry and transport sector</t>
+  </si>
+  <si>
     <t>Scenario1</t>
   </si>
   <si>
@@ -240,120 +276,177 @@
     <t>AccumulatedAnnualDemand</t>
   </si>
   <si>
+    <t>YES_ELAST</t>
+  </si>
+  <si>
+    <t>TRACAR</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
+  </si>
+  <si>
+    <t>TechnologyActivityIncreaseByModeLimit</t>
+  </si>
+  <si>
+    <t>DEP</t>
+  </si>
+  <si>
+    <t>TRADSLCARCUR</t>
+  </si>
+  <si>
+    <t>Capital Costs</t>
+  </si>
+  <si>
+    <t>Capital costs of electric vehicles</t>
+  </si>
+  <si>
+    <t>CapitalCost</t>
+  </si>
+  <si>
+    <t>YES_PROP</t>
+  </si>
+  <si>
+    <t>TRAELCCARCUR</t>
+  </si>
+  <si>
+    <t>Fixed Costs</t>
+  </si>
+  <si>
+    <t>Fixed Cost of electric vehicles technologies</t>
+  </si>
+  <si>
+    <t>FixedCost</t>
+  </si>
+  <si>
+    <t>Capital Cost of ICE vehicles technologies</t>
+  </si>
+  <si>
+    <t>Fixed Cost of ICE vehicles technologies</t>
+  </si>
+  <si>
+    <t>Variable Costs</t>
+  </si>
+  <si>
+    <t>Variable Cost of crops technologies</t>
+  </si>
+  <si>
+    <t>VariableCost</t>
+  </si>
+  <si>
+    <t>LNDMAIHR</t>
+  </si>
+  <si>
+    <t>Fixed Cost of crops technologies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import cost of fuels </t>
+  </si>
+  <si>
     <t>NO</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>1) Multiply final value of time series by the Explored Parameter in each future and then interpolate. 2) Assign the modified parameter back.</t>
+    <t>IMPBIO ; IMPLPG ; IMPHFO ; IMPNGS ; IMPURN ; IMPGSL ; IMPDSL ; IMPKER</t>
+  </si>
+  <si>
+    <t>Coal supply</t>
+  </si>
+  <si>
+    <t>MINCOA</t>
+  </si>
+  <si>
+    <t>Cost of electricity imports</t>
+  </si>
+  <si>
+    <t>PWRTRNIMP</t>
+  </si>
+  <si>
+    <t>Cost of crop imports</t>
+  </si>
+  <si>
+    <t>IMPMAI ; IMPPUL ; IMPSOR ; IMPMTP ; IMPGRO ; IMPWHE ; IMPSUN ; IMPOTC</t>
+  </si>
+  <si>
+    <t>Output Activity Ratio</t>
+  </si>
+  <si>
+    <t>Crop yields</t>
+  </si>
+  <si>
+    <t>OutputActivityRatio</t>
+  </si>
+  <si>
+    <t>LNDMAIHR ; LNDMAIHI ; LNDMAILR ; LNDMAILI ; LNDCANHR ; LNDCANHI ; LNDCANLR ; LNDCANLI ; LNDGROHR ; LNDGROHI ; LNDGROLR ; LNDGROLI ; LNDMTPHR ; LNDMTPHI ; LNDMTPLR ; LNDMTPLI ; LNDOTCHR ; LNDOTCHI ; LNDOTCLR ; LNDOTCLI ; LNDPULHR ; LNDPULHI ; LNDPULLR ; LNDPULLI ; LNDSORHR ; LNDSORHI ; LNDSORLR ; LNDSORLI ; LNDWHEHR ; LNDWHEHI ; LNDWHELR ; LNDWHELI</t>
+  </si>
+  <si>
+    <t>CRPMAI ; CRPCAN ; CRPGRO ; CRPMTP ; CRPOTC ; CRPPUL ; CRPSOR ; CRPWHE</t>
+  </si>
+  <si>
+    <t>Cost of fuel distribution technologies</t>
+  </si>
+  <si>
+    <t>DEMINDELC ; DEMRESELC ; DEMCOMELC ; DEMAGRELC ; DEMTOURELC ; DEMTRAELC</t>
+  </si>
+  <si>
+    <t>User defined constraint</t>
+  </si>
+  <si>
+    <t>Ensure EVs meet a given share of the total capacity</t>
+  </si>
+  <si>
+    <t>UDCMultiplierTotalCapacity</t>
+  </si>
+  <si>
+    <t>YES_ADD</t>
+  </si>
+  <si>
+    <t>2TRACAREVCAP</t>
+  </si>
+  <si>
+    <t>Ensure EVs make up no more than 2% of the total car capacity</t>
+  </si>
+  <si>
+    <t>TRAGSLCARNEW</t>
+  </si>
+  <si>
+    <t>Forces water availability in 2050 to reduce to 75% of the 2020 value.</t>
   </si>
   <si>
     <t>UDCConstant</t>
   </si>
   <si>
-    <t>Capital Costs</t>
-  </si>
-  <si>
-    <t>Capital costs of electric vehicles</t>
-  </si>
-  <si>
-    <t>CapitalCost</t>
-  </si>
-  <si>
-    <t>Fixed Costs</t>
-  </si>
-  <si>
-    <t>Fixed Cost of electric vehicles technologies</t>
-  </si>
-  <si>
-    <t>FixedCost</t>
-  </si>
-  <si>
-    <t>Capital Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>Fixed Cost of ICE vehicles technologies</t>
-  </si>
-  <si>
-    <t>Variable Costs</t>
-  </si>
-  <si>
-    <t>Variable Cost of crops technologies</t>
-  </si>
-  <si>
-    <t>VariableCost</t>
-  </si>
-  <si>
-    <t>LNDMAIHR ; LNDMAIHI ; LNDMAILR ; LNDMAILI ; LNDCANHR ; LNDCANHI ; LNDCANLR ; LNDCANLI ; LNDGROHR ; LNDGROHI ; LNDGROLR ; LNDGROLI ; LNDMTPHR ; LNDMTPHI ; LNDMTPLR ; LNDMTPLI ; LNDOTCHR ; LNDOTCHI ; LNDOTCLR ; LNDOTCLI ; LNDPULHR ; LNDPULHI ; LNDPULLR ; LNDPULLI ; LNDSORHR ; LNDSORHI ; LNDSORLR ; LNDSORLI ; LNDWHEHR ; LNDWHEHI ; LNDWHELR ; LNDWHELI</t>
-  </si>
-  <si>
-    <t>Fixed Cost of crops technologies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Import cost of fuels </t>
-  </si>
-  <si>
-    <t>IMPBIO ; IMPLPG ; IMPHFO ; IMPNGS ; IMPURN ; IMPGSL ; IMPDSL ; IMPKER</t>
-  </si>
-  <si>
-    <t>Cost of electricity imports</t>
-  </si>
-  <si>
-    <t>PWRTRNIMP</t>
-  </si>
-  <si>
-    <t>Cost of crop imports</t>
-  </si>
-  <si>
-    <t>IMPMAI ; IMPPUL ; IMPSOR ; IMPMTP ; IMPGRO ; IMPWHE ; IMPSUN ; IMPOTC</t>
-  </si>
-  <si>
-    <t>Output Activity Ratio</t>
-  </si>
-  <si>
-    <t>Crop yields</t>
-  </si>
-  <si>
-    <t>OutputActivityRatio</t>
-  </si>
-  <si>
-    <t>CRPMAI ; CRPCAN ; CRPGRO ; CRPMTP ; CRPOTC ; CRPPUL ; CRPSOR ; CRPWHE</t>
-  </si>
-  <si>
-    <t>Cost of fuel distribution technologies</t>
-  </si>
-  <si>
-    <t>DEMINDELC ; DEMRESELC ; DEMCOMELC ; DEMAGRELC ; DEMTOURELC ; DEMTRAELC</t>
-  </si>
-  <si>
-    <t>User defined constraint</t>
-  </si>
-  <si>
-    <t>Ensure EVs make up no more than 2% of the total car capacity</t>
-  </si>
-  <si>
-    <t>UDCMultiplierTotalCapacity</t>
-  </si>
-  <si>
-    <t>2TRACAREVCAP</t>
-  </si>
-  <si>
-    <t>Forces water availability in 2050 to reduce to 75% of the 2020 value.</t>
-  </si>
-  <si>
     <t>RESTRICTWAT</t>
   </si>
   <si>
     <t>Collection rate</t>
   </si>
   <si>
+    <t xml:space="preserve">Minimum share of waste that should be collected </t>
+  </si>
+  <si>
     <t>UDCMultiplierActivity</t>
   </si>
   <si>
+    <t>WSTGEN; LWTGEN</t>
+  </si>
+  <si>
+    <t>COLWST; COLLWT</t>
+  </si>
+  <si>
+    <t>Capital costs of renewables</t>
+  </si>
+  <si>
+    <t>PWRSOL001; PWRWND001; PWRBIO001</t>
+  </si>
+  <si>
     <t>Capital costs of the cement industry</t>
   </si>
   <si>
+    <t>INDKILNBIOCCS; INDKILNCOACCS; INDKILNBIO; INDKILNCOA; INDKILNDSL; INDKILNLPG; INDKILNHFO; INDKILNCOA</t>
+  </si>
+  <si>
     <t>Reserve margin</t>
   </si>
   <si>
@@ -363,168 +456,108 @@
     <t>RESMAR</t>
   </si>
   <si>
+    <t>Demand growth in the agriculture sector</t>
+  </si>
+  <si>
+    <t>LVSSHP</t>
+  </si>
+  <si>
     <t>Cattle population demand growth</t>
   </si>
   <si>
     <t>LVSCTL</t>
   </si>
   <si>
+    <t>Activity Limit</t>
+  </si>
+  <si>
+    <t>Electricity import availability</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>TotalTechnologyAnnualActivityUpperLimit</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>YearSplit</t>
+  </si>
+  <si>
+    <t>DiscountRate</t>
+  </si>
+  <si>
+    <t>DiscountRateIdv</t>
+  </si>
+  <si>
+    <t>TradeRoute</t>
+  </si>
+  <si>
+    <t>DepreciationMethod</t>
+  </si>
+  <si>
+    <t>Conversionls</t>
+  </si>
+  <si>
+    <t>Conversionld</t>
+  </si>
+  <si>
+    <t>Conversionlh</t>
+  </si>
+  <si>
+    <t>DaySplit</t>
+  </si>
+  <si>
+    <t>DaysInDayType</t>
+  </si>
+  <si>
+    <t>SpecifiedAnnualDemand</t>
+  </si>
+  <si>
+    <t>SpecifiedDemandProfile</t>
+  </si>
+  <si>
+    <t>CapacityToActivityUnit</t>
+  </si>
+  <si>
+    <t>CapitalRecoveryFactor</t>
+  </si>
+  <si>
+    <t>CapacityOfOneTechnologyUnit</t>
+  </si>
+  <si>
+    <t>CapacityFactor</t>
+  </si>
+  <si>
+    <t>AvailabilityFactor</t>
+  </si>
+  <si>
+    <t>OperationalLife</t>
+  </si>
+  <si>
+    <t>ResidualCapacity</t>
+  </si>
+  <si>
+    <t>InputActivityRatio</t>
+  </si>
+  <si>
+    <t>InputToNewCapacityRatio</t>
+  </si>
+  <si>
+    <t>InputToTotalCapacityRatio</t>
+  </si>
+  <si>
+    <t>PvAnnuity</t>
+  </si>
+  <si>
+    <t>CapitalCostStorage</t>
+  </si>
+  <si>
     <t>TotalAnnualMaxCapacity</t>
   </si>
   <si>
-    <t>Activity Limit</t>
-  </si>
-  <si>
-    <t>Electricity import availability</t>
-  </si>
-  <si>
-    <t>Step</t>
-  </si>
-  <si>
-    <t>TotalTechnologyAnnualActivityUpperLimit</t>
-  </si>
-  <si>
-    <t>Number_of_Runs</t>
-  </si>
-  <si>
-    <t>Scenario_to_Reproduce</t>
-  </si>
-  <si>
-    <t>Experiment_ID</t>
-  </si>
-  <si>
-    <t>Parallel_Use</t>
-  </si>
-  <si>
-    <t>Timeslices_model</t>
-  </si>
-  <si>
-    <t>Run_Base_Future</t>
-  </si>
-  <si>
-    <t>Run_RDM</t>
-  </si>
-  <si>
-    <t>Solver</t>
-  </si>
-  <si>
-    <t>OSeMOSYS_Model_Name</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>EV_Conventional_Patterns</t>
-  </si>
-  <si>
-    <t>EV_Electric_Pattern</t>
-  </si>
-  <si>
-    <t>EV_UDCs</t>
-  </si>
-  <si>
-    <t>Experiment</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>cplex</t>
-  </si>
-  <si>
-    <t>model.v.5.4.txt</t>
-  </si>
-  <si>
-    <t>BWA</t>
-  </si>
-  <si>
-    <t>DSL;DSH;GSL</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>2TRACAREVCAP;2TRAMCYEVCAP;2TRABUSEVCAP;2TRAMNBEVCAP;2TRALTREVCAP;2TRAMTREVCAP;2TRAHTREVCAP</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>YearSplit</t>
-  </si>
-  <si>
-    <t>DiscountRate</t>
-  </si>
-  <si>
-    <t>DiscountRateIdv</t>
-  </si>
-  <si>
-    <t>TradeRoute</t>
-  </si>
-  <si>
-    <t>DepreciationMethod</t>
-  </si>
-  <si>
-    <t>Conversionls</t>
-  </si>
-  <si>
-    <t>Conversionld</t>
-  </si>
-  <si>
-    <t>Conversionlh</t>
-  </si>
-  <si>
-    <t>DaySplit</t>
-  </si>
-  <si>
-    <t>DaysInDayType</t>
-  </si>
-  <si>
-    <t>SpecifiedAnnualDemand</t>
-  </si>
-  <si>
-    <t>SpecifiedDemandProfile</t>
-  </si>
-  <si>
-    <t>CapacityToActivityUnit</t>
-  </si>
-  <si>
-    <t>CapitalRecoveryFactor</t>
-  </si>
-  <si>
-    <t>CapacityOfOneTechnologyUnit</t>
-  </si>
-  <si>
-    <t>CapacityFactor</t>
-  </si>
-  <si>
-    <t>AvailabilityFactor</t>
-  </si>
-  <si>
-    <t>OperationalLife</t>
-  </si>
-  <si>
-    <t>ResidualCapacity</t>
-  </si>
-  <si>
-    <t>InputActivityRatio</t>
-  </si>
-  <si>
-    <t>InputToNewCapacityRatio</t>
-  </si>
-  <si>
-    <t>InputToTotalCapacityRatio</t>
-  </si>
-  <si>
-    <t>PvAnnuity</t>
-  </si>
-  <si>
-    <t>CapitalCostStorage</t>
-  </si>
-  <si>
     <t>TotalAnnualMinCapacity</t>
   </si>
   <si>
@@ -576,9 +609,6 @@
     <t>ResidualStorageCapacity</t>
   </si>
   <si>
-    <t>TechnologyActivityIncreaseByModeLimit</t>
-  </si>
-  <si>
     <t>TechnologyActivityDecreaseByModeLimit</t>
   </si>
   <si>
@@ -754,76 +784,13 @@
   </si>
   <si>
     <t>TotalDiscountedStorageCost</t>
-  </si>
-  <si>
-    <t>YES_ELAST</t>
-  </si>
-  <si>
-    <t>YES_ADD</t>
-  </si>
-  <si>
-    <t>INDKILNBIOCCS; INDKILNCOACCS; INDKILNBIO; INDKILNCOA; INDKILNDSL; INDKILNLPG; INDKILNHFO; INDKILNCOA</t>
-  </si>
-  <si>
-    <t>TRAELCCARCUR</t>
-  </si>
-  <si>
-    <t>YES_PROP</t>
-  </si>
-  <si>
-    <t>DEP</t>
-  </si>
-  <si>
-    <t>TRADSLCARCUR</t>
-  </si>
-  <si>
-    <t>Demand growth in the buildings, industry and transport sector</t>
-  </si>
-  <si>
-    <t>TRACAR</t>
-  </si>
-  <si>
-    <t>LNDMAIHR</t>
-  </si>
-  <si>
-    <t>Coal supply</t>
-  </si>
-  <si>
-    <t>MINCOA</t>
-  </si>
-  <si>
-    <t>Ensure EVs meet a given share of the total capacity</t>
-  </si>
-  <si>
-    <t>TRAGSLCARNEW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum share of waste that should be collected </t>
-  </si>
-  <si>
-    <t>WSTGEN; LWTGEN</t>
-  </si>
-  <si>
-    <t>COLWST; COLLWT</t>
-  </si>
-  <si>
-    <t>Capital costs of renewables</t>
-  </si>
-  <si>
-    <t>PWRSOL001; PWRWND001; PWRBIO001</t>
-  </si>
-  <si>
-    <t>Demand growth in the agriculture sector</t>
-  </si>
-  <si>
-    <t>LVSSHP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -900,19 +867,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1588,92 +1542,93 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{085A3DD8-2D99-42E9-A4DB-6F2A902CF2BA}">
-  <dimension ref="A1:O39"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="15" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" style="15" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" style="15" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" style="15" customWidth="1"/>
     <col min="3" max="3" width="44" style="16" customWidth="1"/>
-    <col min="4" max="4" width="24.42578125" style="19" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" style="19" customWidth="1"/>
-    <col min="6" max="7" width="32.140625" style="19" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" style="19" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" style="19" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="27.44140625" style="19" customWidth="1"/>
+    <col min="6" max="7" width="32.109375" style="19" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" style="19" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" style="19" customWidth="1"/>
     <col min="10" max="10" width="54" style="15" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="79.7109375" style="16" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" style="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="79.6640625" style="16" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="49" style="20" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="45.85546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="45.88671875" style="19" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="44" style="20" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.85546875" style="27"/>
+    <col min="16" max="16" width="8.88671875" style="27" customWidth="1"/>
+    <col min="17" max="16384" width="8.88671875" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="15" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="K1" s="25" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="L1" s="18" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="O1" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33">
         <v>1</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C2" s="34" t="s">
-        <v>199</v>
+        <v>39</v>
       </c>
       <c r="D2" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E2" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F2" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G2" s="33">
         <v>2026</v>
@@ -1685,43 +1640,43 @@
         <v>1.5</v>
       </c>
       <c r="J2" s="33" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="K2" s="35" t="s">
-        <v>192</v>
+        <v>44</v>
       </c>
       <c r="L2" s="36" t="s">
-        <v>200</v>
+        <v>45</v>
       </c>
       <c r="M2" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N2" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O2" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" s="40" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" s="40" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="37">
         <f t="shared" ref="A3:A26" si="0">A2+1</f>
         <v>2</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C3" s="34" t="s">
-        <v>199</v>
+        <v>39</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G3" s="37">
         <v>2026</v>
@@ -1733,43 +1688,43 @@
         <v>2</v>
       </c>
       <c r="J3" s="37" t="s">
-        <v>132</v>
+        <v>48</v>
       </c>
       <c r="K3" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L3" s="39" t="s">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="M3" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N3" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O3" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="33">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C4" s="34" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G4" s="33">
         <v>2026</v>
@@ -1781,41 +1736,41 @@
         <v>1.5</v>
       </c>
       <c r="J4" s="33" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="K4" s="35" t="s">
-        <v>196</v>
+        <v>54</v>
       </c>
       <c r="L4" s="41" t="s">
-        <v>195</v>
+        <v>55</v>
       </c>
       <c r="M4" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N4" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O4" s="42"/>
     </row>
-    <row r="5" spans="1:15" s="28" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" s="28" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="D5" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G5" s="37">
         <v>2026</v>
@@ -1827,43 +1782,43 @@
         <v>1.5</v>
       </c>
       <c r="J5" s="37" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L5" s="43" t="s">
-        <v>195</v>
+        <v>55</v>
       </c>
       <c r="M5" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N5" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O5" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" s="15" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" s="15" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="33">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G6" s="33">
         <v>2026</v>
@@ -1875,43 +1830,43 @@
         <v>1.5</v>
       </c>
       <c r="J6" s="33" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="K6" s="35" t="s">
-        <v>196</v>
+        <v>54</v>
       </c>
       <c r="L6" s="34" t="s">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="M6" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N6" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O6" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" s="44" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" s="44" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="37">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G7" s="37">
         <v>2026</v>
@@ -1923,43 +1878,43 @@
         <v>1.5</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K7" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L7" s="39" t="s">
-        <v>198</v>
+        <v>50</v>
       </c>
       <c r="M7" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N7" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O7" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="33">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G8" s="33">
         <v>2026</v>
@@ -1971,43 +1926,43 @@
         <v>1.5</v>
       </c>
       <c r="J8" s="34" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="K8" s="35" t="s">
-        <v>196</v>
+        <v>54</v>
       </c>
       <c r="L8" s="45" t="s">
-        <v>201</v>
+        <v>64</v>
       </c>
       <c r="M8" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N8" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O8" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" s="40" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" s="40" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="37">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C9" s="39" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G9" s="37">
         <v>2026</v>
@@ -2019,43 +1974,43 @@
         <v>1.5</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="K9" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L9" s="46" t="s">
-        <v>201</v>
+        <v>64</v>
       </c>
       <c r="M9" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N9" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O9" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G10" s="15">
         <v>2026</v>
@@ -2067,43 +2022,43 @@
         <v>1.5</v>
       </c>
       <c r="J10" s="16" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="K10" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="M10" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O10" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>202</v>
+        <v>69</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G11" s="15">
         <v>2026</v>
@@ -2115,43 +2070,43 @@
         <v>1.5</v>
       </c>
       <c r="J11" s="16" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="K11" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>203</v>
+        <v>70</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O11" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G12" s="15">
         <v>2026</v>
@@ -2163,43 +2118,43 @@
         <v>1.5</v>
       </c>
       <c r="J12" s="16" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="K12" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L12" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N12" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="O12" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="M12" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="N12" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="O12" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="16" t="s">
+      <c r="E13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>17</v>
-      </c>
       <c r="F13" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G13" s="15">
         <v>2026</v>
@@ -2211,43 +2166,43 @@
         <v>1.5</v>
       </c>
       <c r="J13" s="16" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="K13" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L13" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N13" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="O13" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="15" t="s">
         <v>42</v>
-      </c>
-      <c r="M13" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="N13" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="O13" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>18</v>
       </c>
       <c r="G14" s="15">
         <v>2026</v>
@@ -2259,43 +2214,43 @@
         <v>1.5</v>
       </c>
       <c r="J14" s="16" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="K14" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L14" s="16" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="N14" s="16" t="s">
-        <v>21</v>
+        <v>79</v>
+      </c>
+      <c r="N14" s="16">
+        <v>1</v>
       </c>
       <c r="O14" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="15">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G15" s="15">
         <v>2026</v>
@@ -2307,37 +2262,37 @@
         <v>1.5</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="K15" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L15" s="16" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="O15" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B16" s="33" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="C16" s="34" t="s">
-        <v>204</v>
+        <v>83</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E16" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G16" s="33">
         <v>2026</v>
@@ -2349,43 +2304,43 @@
         <v>1</v>
       </c>
       <c r="J16" s="33" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="K16" s="35" t="s">
-        <v>193</v>
+        <v>85</v>
       </c>
       <c r="L16" s="34" t="s">
-        <v>195</v>
+        <v>55</v>
       </c>
       <c r="M16" s="34" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="N16" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O16" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" s="29" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" s="29" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="33">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="C17" s="39" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F17" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G17" s="37">
         <v>2026</v>
@@ -2397,43 +2352,43 @@
         <v>1</v>
       </c>
       <c r="J17" s="37" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="K17" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L17" s="39" t="s">
-        <v>205</v>
+        <v>88</v>
       </c>
       <c r="M17" s="39" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="N17" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O17" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G18" s="15">
         <v>2026</v>
@@ -2445,43 +2400,43 @@
         <v>1.5</v>
       </c>
       <c r="J18" s="15" t="s">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="K18" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N18" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O18" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:15" s="48" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" s="48" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="48">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C19" s="50" t="s">
-        <v>206</v>
+        <v>93</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E19" s="51" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G19" s="48">
         <v>2026</v>
@@ -2493,43 +2448,43 @@
         <v>1.5</v>
       </c>
       <c r="J19" s="49" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="K19" s="52" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L19" s="50" t="s">
-        <v>207</v>
+        <v>95</v>
       </c>
       <c r="M19" s="50" t="s">
-        <v>208</v>
+        <v>96</v>
       </c>
       <c r="N19" s="53" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O19" s="53" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="15">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>209</v>
+        <v>97</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G20" s="15">
         <v>2026</v>
@@ -2541,43 +2496,43 @@
         <v>1.5</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="K20" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N20" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="O20" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="15">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="L20" s="16" t="s">
-        <v>210</v>
-      </c>
-      <c r="M20" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="N20" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="O20" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
       <c r="B21" s="15" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G21" s="15">
         <v>2026</v>
@@ -2589,43 +2544,43 @@
         <v>1.5</v>
       </c>
       <c r="J21" s="15" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="K21" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L21" s="16" t="s">
-        <v>194</v>
+        <v>100</v>
       </c>
       <c r="M21" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="N21" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="O21" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="15">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="N21" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="O21" s="16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
       <c r="B22" s="15" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G22" s="15">
         <v>2026</v>
@@ -2637,43 +2592,43 @@
         <v>1.1299999999999999</v>
       </c>
       <c r="J22" s="15" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="K22" s="26" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L22" s="54" t="s">
-        <v>59</v>
+        <v>102</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="N22" s="16" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O22" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" s="55" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="33">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" s="55" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" s="33">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
       <c r="B23" s="33" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C23" s="34" t="s">
-        <v>211</v>
+        <v>104</v>
       </c>
       <c r="D23" s="33" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F23" s="33" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G23" s="33">
         <v>2026</v>
@@ -2685,43 +2640,43 @@
         <v>1.5</v>
       </c>
       <c r="J23" s="33" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="K23" s="35" t="s">
-        <v>192</v>
+        <v>44</v>
       </c>
       <c r="L23" s="34" t="s">
-        <v>212</v>
+        <v>105</v>
       </c>
       <c r="M23" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N23" s="34" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O23" s="34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" s="40" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" s="40" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="33">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B24" s="37" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C24" s="39" t="s">
-        <v>211</v>
+        <v>104</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E24" s="37" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G24" s="37">
         <v>2026</v>
@@ -2733,43 +2688,43 @@
         <v>2</v>
       </c>
       <c r="J24" s="37" t="s">
-        <v>132</v>
+        <v>48</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>197</v>
+        <v>49</v>
       </c>
       <c r="L24" s="46" t="s">
-        <v>201</v>
+        <v>64</v>
       </c>
       <c r="M24" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N24" s="39" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O24" s="39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" s="55" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" s="55" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="48">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B25" s="48" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="C25" s="53" t="s">
-        <v>61</v>
+        <v>106</v>
       </c>
       <c r="D25" s="48" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E25" s="48" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="F25" s="48" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G25" s="48">
         <v>2026</v>
@@ -2781,43 +2736,43 @@
         <v>1</v>
       </c>
       <c r="J25" s="48" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="K25" s="57" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="L25" s="53" t="s">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="M25" s="53" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N25" s="53" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O25" s="53" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" ht="60" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="15">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B26" s="30" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>65</v>
+        <v>109</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E26" s="30" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G26" s="30">
         <v>2027</v>
@@ -2829,141 +2784,140 @@
         <v>20</v>
       </c>
       <c r="J26" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="K26" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="K26" s="32" t="s">
-        <v>20</v>
-      </c>
       <c r="L26" s="31" t="s">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="M26" s="23" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="N26" s="23" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="O26" s="23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25"/>
-    <row r="33" x14ac:dyDescent="0.25"/>
-    <row r="34" x14ac:dyDescent="0.25"/>
-    <row r="35" x14ac:dyDescent="0.25"/>
-    <row r="36" x14ac:dyDescent="0.25"/>
-    <row r="37" x14ac:dyDescent="0.25"/>
-    <row r="38" x14ac:dyDescent="0.25"/>
-    <row r="39" x14ac:dyDescent="0.25"/>
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O1" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}"/>
+  <autoFilter ref="A1:O1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="15.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr defaultColWidth="15.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>70</v>
+        <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>71</v>
+        <v>3</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>74</v>
+        <v>6</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>79</v>
+        <v>11</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="N1" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="120.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>81</v>
+        <v>15</v>
       </c>
       <c r="C2" s="5">
         <v>1</v>
       </c>
       <c r="D2" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E2" s="9">
         <v>8</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>83</v>
+        <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="J2" s="21" t="s">
-        <v>86</v>
+        <v>19</v>
       </c>
       <c r="K2" s="21" t="s">
-        <v>87</v>
+        <v>20</v>
       </c>
       <c r="L2" s="21" t="s">
-        <v>88</v>
+        <v>21</v>
       </c>
       <c r="M2" s="24" t="s">
-        <v>89</v>
+        <v>22</v>
+      </c>
+      <c r="N2" s="21">
+        <v>2</v>
+      </c>
+      <c r="O2" s="24">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -2973,248 +2927,248 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:BG12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BG5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="21" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="28.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="18" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="23" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="29.42578125" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="33.88671875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="22.88671875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="22" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="18" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="23.109375" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="38" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="38.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="54" width="35.85546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="54" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="58" max="58" width="26" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="7.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="H1" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="J1" t="s">
+        <v>121</v>
+      </c>
+      <c r="K1" t="s">
+        <v>122</v>
+      </c>
+      <c r="L1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M1" t="s">
+        <v>124</v>
+      </c>
+      <c r="N1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>127</v>
+      </c>
+      <c r="R1" t="s">
+        <v>128</v>
+      </c>
+      <c r="S1" t="s">
+        <v>129</v>
+      </c>
+      <c r="T1" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="U1" t="s">
+        <v>131</v>
+      </c>
+      <c r="V1" t="s">
+        <v>132</v>
+      </c>
+      <c r="W1" t="s">
+        <v>133</v>
+      </c>
+      <c r="X1" t="s">
+        <v>134</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z1" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>139</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>140</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>141</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>142</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>143</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>144</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AO1" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>147</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AR1" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="AS1" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="AT1" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AV1" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>155</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>156</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>157</v>
+      </c>
+      <c r="BC1" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="B1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E1" s="13" t="s">
+      <c r="BD1" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="F1" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="J1" t="s">
-        <v>99</v>
-      </c>
-      <c r="K1" t="s">
-        <v>100</v>
-      </c>
-      <c r="L1" t="s">
-        <v>101</v>
-      </c>
-      <c r="M1" t="s">
-        <v>102</v>
-      </c>
-      <c r="N1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O1" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>105</v>
-      </c>
-      <c r="R1" t="s">
-        <v>106</v>
-      </c>
-      <c r="S1" t="s">
-        <v>107</v>
-      </c>
-      <c r="T1" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="U1" t="s">
-        <v>109</v>
-      </c>
-      <c r="V1" t="s">
-        <v>110</v>
-      </c>
-      <c r="W1" t="s">
-        <v>111</v>
-      </c>
-      <c r="X1" t="s">
-        <v>112</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>45</v>
-      </c>
-      <c r="Z1" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>63</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>115</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>116</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>117</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>118</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>119</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>120</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>121</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>122</v>
-      </c>
-      <c r="AO1" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>124</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>125</v>
-      </c>
-      <c r="AR1" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="AS1" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="AT1" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>129</v>
-      </c>
-      <c r="AV1" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>131</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>132</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>133</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>134</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>135</v>
-      </c>
-      <c r="BC1" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="BD1" s="14" t="s">
-        <v>56</v>
-      </c>
       <c r="BE1" s="14" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="BF1" s="14" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="BG1" s="13" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="2" spans="1:59" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="B2">
         <f t="shared" ref="B2:AQ2" si="0">+COUNTA(B3:B1048576)</f>
@@ -3449,183 +3403,183 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:59" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:59" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="J3" t="s">
-        <v>141</v>
+        <v>163</v>
       </c>
       <c r="K3" t="s">
-        <v>142</v>
+        <v>164</v>
       </c>
       <c r="L3" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="M3" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="N3" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="O3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="P3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="Q3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="R3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="S3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="T3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="U3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="V3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="W3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="X3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="Y3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="Z3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="AA3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AB3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AC3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AD3" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AE3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AF3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AG3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AH3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AI3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AJ3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AK3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AL3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AM3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AN3" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="AO3" s="13" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="AP3" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="AQ3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AR3" s="13" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AS3" s="13" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AT3" s="13" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AU3" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AV3" s="13" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="AW3" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AX3" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AY3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="AZ3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BA3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BB3" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BC3" s="14" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="BD3" s="14" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BE3" s="14" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BF3" s="14" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="BG3" s="13" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:59" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="4" spans="1:59" x14ac:dyDescent="0.3">
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
@@ -3634,74 +3588,74 @@
       <c r="H4" s="13"/>
       <c r="I4" s="13"/>
       <c r="M4" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="O4" s="13"/>
       <c r="P4" s="13"/>
       <c r="R4" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
       <c r="T4" s="13"/>
       <c r="V4" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="W4" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="X4" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="Y4" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="Z4" s="13"/>
       <c r="AB4" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AM4" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="AO4" s="13"/>
       <c r="AQ4" t="s">
-        <v>146</v>
+        <v>168</v>
       </c>
       <c r="AR4" s="13" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AS4" s="13" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AT4" s="13"/>
       <c r="AV4" s="13" t="s">
-        <v>145</v>
+        <v>167</v>
       </c>
       <c r="AY4" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AZ4" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="BA4" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="BB4" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="BC4" s="14"/>
       <c r="BD4" s="14" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="BE4" s="14" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="BF4" s="14" t="s">
-        <v>147</v>
+        <v>169</v>
       </c>
       <c r="BG4" s="13" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="5" spans="1:59" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:59" x14ac:dyDescent="0.3">
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
@@ -3713,24 +3667,24 @@
       <c r="P5" s="13"/>
       <c r="T5" s="13"/>
       <c r="V5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="Y5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="Z5" s="13"/>
       <c r="AM5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AO5" s="13"/>
       <c r="AQ5" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AR5" s="13" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AS5" s="13" t="s">
-        <v>148</v>
+        <v>170</v>
       </c>
       <c r="AT5" s="13"/>
       <c r="AV5" s="13"/>
@@ -3739,11 +3693,6 @@
       <c r="BE5" s="14"/>
       <c r="BF5" s="14"/>
       <c r="BG5" s="13"/>
-    </row>
-    <row r="12" spans="1:59" x14ac:dyDescent="0.25">
-      <c r="AY12">
-        <v>89888090</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3754,248 +3703,248 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.44140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>149</v>
+        <v>171</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>176</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>178</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>210</v>
+      </c>
+      <c r="B38" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>188</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
30-03 scenarios with interface table running
</commit_message>
<xml_diff>
--- a/src/Interface_RDM.xlsx
+++ b/src/Interface_RDM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RDM\github_RDM\osemosys-rdm\src\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\osemosys-rdm\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3370E254-041B-4367-8031-C64CA627B5CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D869C37-6B1A-4985-A296-4DD9909EC76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="727" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -178,7 +178,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2344" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2453" uniqueCount="317">
   <si>
     <t>X_Num</t>
   </si>
@@ -1122,23 +1122,20 @@
     <t>TRACAR</t>
   </si>
   <si>
-    <t>TRAMNB</t>
-  </si>
-  <si>
     <t>TRALTR</t>
   </si>
   <si>
+    <t>TRAHTR</t>
+  </si>
+  <si>
     <t>TRAMTR</t>
-  </si>
-  <si>
-    <t>TRAHTR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1205,6 +1202,12 @@
       <color theme="4"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1762,7 +1765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{085A3DD8-2D99-42E9-A4DB-6F2A902CF2BA}">
-  <dimension ref="A1:O197"/>
+  <dimension ref="A1:O208"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" style="19" customWidth="1"/>
@@ -10833,11 +10836,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="194" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A194" s="19">
-        <v>196</v>
-      </c>
-      <c r="B194" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="B194" s="25" t="s">
         <v>15</v>
       </c>
       <c r="C194" s="21" t="s">
@@ -10846,45 +10849,45 @@
       <c r="D194" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="E194" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F194" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G194" s="19">
-        <v>2026</v>
-      </c>
-      <c r="H194" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="I194" s="19">
-        <v>1</v>
-      </c>
-      <c r="J194" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="K194" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="L194" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="M194" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="N194" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="O194" s="21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="195" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E194" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F194" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G194" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H194" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I194" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J194" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K194" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L194" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="M194" s="27">
+        <v>1</v>
+      </c>
+      <c r="N194" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O194" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="195" spans="1:15" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A195" s="19">
-        <v>201</v>
-      </c>
-      <c r="B195" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="B195" s="25" t="s">
         <v>15</v>
       </c>
       <c r="C195" s="21" t="s">
@@ -10893,45 +10896,45 @@
       <c r="D195" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="E195" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F195" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G195" s="19">
-        <v>2026</v>
-      </c>
-      <c r="H195" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="I195" s="19">
-        <v>1.2</v>
-      </c>
-      <c r="J195" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="K195" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="L195" s="22" t="s">
-        <v>315</v>
-      </c>
-      <c r="M195" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="N195" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="O195" s="21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="196" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E195" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F195" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G195" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H195" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I195" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J195" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K195" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L195" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="M195" s="27">
+        <v>1</v>
+      </c>
+      <c r="N195" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O195" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="196" spans="1:15" s="25" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A196" s="19">
-        <v>205</v>
-      </c>
-      <c r="B196" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="B196" s="25" t="s">
         <v>15</v>
       </c>
       <c r="C196" s="21" t="s">
@@ -10940,43 +10943,43 @@
       <c r="D196" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="E196" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="F196" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G196" s="19">
-        <v>2026</v>
-      </c>
-      <c r="H196" s="19">
-        <v>0.5</v>
-      </c>
-      <c r="I196" s="19">
-        <v>1.2</v>
-      </c>
-      <c r="J196" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="K196" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="L196" s="22" t="s">
-        <v>316</v>
-      </c>
-      <c r="M196" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="N196" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="O196" s="21" t="s">
+      <c r="E196" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F196" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G196" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H196" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I196" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J196" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K196" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L196" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="M196" s="27">
+        <v>1</v>
+      </c>
+      <c r="N196" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O196" s="27" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="197" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="19">
-        <v>209</v>
+        <v>196</v>
       </c>
       <c r="B197" s="19" t="s">
         <v>15</v>
@@ -11006,10 +11009,10 @@
         <v>18</v>
       </c>
       <c r="K197" s="23" t="s">
-        <v>19</v>
+        <v>311</v>
       </c>
       <c r="L197" s="22" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="M197" s="21" t="s">
         <v>20</v>
@@ -11018,11 +11021,529 @@
         <v>20</v>
       </c>
       <c r="O197" s="21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="198" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A198" s="19">
+        <v>197</v>
+      </c>
+      <c r="B198" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C198" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D198" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E198" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F198" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G198" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H198" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I198" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J198" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K198" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L198" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="M198" s="27">
+        <v>1</v>
+      </c>
+      <c r="N198" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O198" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="199" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A199" s="19">
+        <v>198</v>
+      </c>
+      <c r="B199" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C199" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D199" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E199" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F199" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G199" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H199" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I199" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J199" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K199" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L199" s="27" t="s">
+        <v>301</v>
+      </c>
+      <c r="M199" s="27">
+        <v>1</v>
+      </c>
+      <c r="N199" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O199" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="200" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A200" s="19">
+        <v>199</v>
+      </c>
+      <c r="B200" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C200" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D200" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E200" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F200" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G200" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H200" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I200" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J200" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K200" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L200" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="M200" s="27">
+        <v>1</v>
+      </c>
+      <c r="N200" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O200" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="201" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A201" s="19">
+        <v>200</v>
+      </c>
+      <c r="B201" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C201" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D201" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E201" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F201" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G201" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H201" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="I201" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="J201" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="K201" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="L201" s="22" t="s">
+        <v>315</v>
+      </c>
+      <c r="M201" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="N201" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="O201" s="21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="202" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A202" s="19">
+        <v>201</v>
+      </c>
+      <c r="B202" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C202" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D202" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E202" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F202" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G202" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H202" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I202" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J202" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K202" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L202" s="27" t="s">
+        <v>196</v>
+      </c>
+      <c r="M202" s="27">
+        <v>1</v>
+      </c>
+      <c r="N202" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O202" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="203" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A203" s="19">
+        <v>202</v>
+      </c>
+      <c r="B203" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C203" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D203" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E203" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F203" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G203" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H203" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I203" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J203" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K203" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L203" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="M203" s="27">
+        <v>1</v>
+      </c>
+      <c r="N203" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O203" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="204" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A204" s="19">
+        <v>203</v>
+      </c>
+      <c r="B204" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C204" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D204" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E204" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F204" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G204" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H204" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I204" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J204" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K204" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L204" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="M204" s="27">
+        <v>1</v>
+      </c>
+      <c r="N204" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O204" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="205" spans="1:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A205" s="19">
+        <v>204</v>
+      </c>
+      <c r="B205" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C205" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D205" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E205" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F205" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G205" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H205" s="19">
+        <v>0.5</v>
+      </c>
+      <c r="I205" s="19">
+        <v>1.2</v>
+      </c>
+      <c r="J205" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="K205" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="L205" s="22" t="s">
+        <v>316</v>
+      </c>
+      <c r="M205" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="N205" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="O205" s="21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="206" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A206" s="19">
+        <v>205</v>
+      </c>
+      <c r="B206" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C206" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D206" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E206" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F206" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G206" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H206" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I206" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J206" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K206" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L206" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="M206" s="27">
+        <v>1</v>
+      </c>
+      <c r="N206" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O206" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="207" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A207" s="19">
+        <v>206</v>
+      </c>
+      <c r="B207" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C207" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D207" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E207" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F207" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G207" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H207" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I207" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J207" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K207" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L207" s="27" t="s">
+        <v>306</v>
+      </c>
+      <c r="M207" s="27">
+        <v>1</v>
+      </c>
+      <c r="N207" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O207" s="27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="208" spans="1:15" s="25" customFormat="1" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A208" s="19">
+        <v>207</v>
+      </c>
+      <c r="B208" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C208" s="21" t="s">
+        <v>178</v>
+      </c>
+      <c r="D208" s="19" t="s">
+        <v>274</v>
+      </c>
+      <c r="E208" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F208" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G208" s="25">
+        <v>2026</v>
+      </c>
+      <c r="H208" s="25">
+        <v>0.1</v>
+      </c>
+      <c r="I208" s="25">
+        <v>1.5</v>
+      </c>
+      <c r="J208" s="25" t="s">
+        <v>117</v>
+      </c>
+      <c r="K208" s="26" t="s">
+        <v>192</v>
+      </c>
+      <c r="L208" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="M208" s="27">
+        <v>1</v>
+      </c>
+      <c r="N208" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="O208" s="27" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O2" xr:uid="{95B5B787-8749-47D9-9D7A-FB53FE5A30D3}"/>
+  <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
@@ -11103,7 +11624,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="8">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E2" s="9">
         <v>8</v>

</xml_diff>